<commit_message>
Add Documentation tab; rename Wife to Spouse for reusability
New first tab covers the SRR-shield motivation, how the four tabs fit
together, a quarterly operating checklist, the color legend, and a
glossary -- meant for family members and an advisor who weren't part of
building this.

Also renames "Wife" labels/pronouns to "Spouse"/"Their" throughout
Account_Tracker and the Emergency Liquidity Protocol text so the workbook
isn't tied to one household's specific configuration.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/household_portfolio_engine.xlsx
+++ b/household_portfolio_engine.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables_And_Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account_Tracker" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The_Refill_Engine" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables_And_Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account_Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The_Refill_Engine" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -42,21 +43,21 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -65,14 +66,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0044546A"/>
-        <bgColor rgb="0044546A"/>
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-        <bgColor rgb="001F3864"/>
+        <fgColor rgb="0044546A"/>
+        <bgColor rgb="0044546A"/>
       </patternFill>
     </fill>
     <fill>
@@ -85,6 +86,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="00DCE6F1"/>
         <bgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4E4"/>
+        <bgColor rgb="00FCE4E4"/>
       </patternFill>
     </fill>
   </fills>
@@ -128,31 +147,50 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -161,7 +199,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -571,6 +608,400 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HOUSEHOLD PORTFOLIO ENGINE — DOCUMENTATION &amp; USER GUIDE</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>WHY THIS SPREADSHEET EXISTS</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="83" customHeight="1">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>This workbook manages a two-bucket, decumulation-phase retirement income strategy built to protect the household from Sequence-of-Returns Risk (SRR) -- the danger that a market downturn early in retirement forces the sale of depreciated stocks to cover monthly living expenses, permanently damaging the portfolio's ability to recover. The strategy rests on three ideas, described below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="83" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>1. The TSP G Fund as a "free lunch" cash vault. By law, the G Fund earns the yield of intermediate- to long-term Treasuries while never losing principal value and staying instantly liquid. It serves as the household's operating cash account -- monthly bills are paid straight out of it, so equities are never sold to cover routine expenses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98" customHeight="1">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2. A dynamic Refill Engine, not a fixed withdrawal rate. Instead of a static 4%-rule, this workbook tracks a real-growth hurdle (COLA layered on a fixed real-growth baseline) year over year. When actual household wealth clears that hurdle, it's safe to harvest equity gains and roll them back into the G Fund to top the shield back up. When wealth falls short, all equity sales freeze and the G Fund alone absorbs spending, giving stocks time to recover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="83" customHeight="1">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>3. Asset location by account. Safe, fixed-income assets are deliberately concentrated in accounts built for stability (the TSP G Fund, a spouse's workplace plan), while private IRAs hold the aggressive growth positions and serve as Roth-conversion conduits -- keeping each spouse's accounts doing the job they're best suited for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>HOW THE FOUR TABS WORK TOGETHER</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="53" customHeight="1">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Documentation (this tab) -- Motivation, how-to, a quarterly checklist, the color legend, and a glossary. Nothing here feeds any formula; it's for the humans using the sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="68" customHeight="1">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Variables_And_Log -- Where you log the two things that change constantly: the actual Social Security/Federal COLA each year, and every month's actual TSP -&gt; checking payment. Everything else on this tab is a formula built from those two inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="68" customHeight="1">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Account_Tracker -- A snapshot of every account's live balance, updated by hand whenever you check statements (aim for at least quarterly). This is the single source of truth for household net worth that every other tab's formulas reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="98" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>The_Refill_Engine -- The decision-making tab. The Quarterly Refill Engine table is the headline output -- each quarter it tells you how much (if anything) to move from a private pre-tax account into the TSP G Fund. Below that, the Annual SRR Hurdle Model is the strategic gauge that decides GOOD vs. POOR for the year, and the Emergency Liquidity Protocol tells you, in a full-blown crisis, exactly which account to draw from next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>YOUR QUARTERLY CHECKLIST</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n"/>
+    </row>
+    <row r="16" ht="23" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Update Account_Tracker with current balances from your statements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Confirm Variables_And_Log has this quarter's three monthly TSP payments logged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Open The_Refill_Engine and find this quarter's row in the Quarterly Refill Engine table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Check the "Recommended Transfer This Quarter" cell. If it's $0, do nothing -- the shield is intact or the market hasn't cleared its hurdle yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>If it's a positive number, execute a pre-tax rollover of that amount from your Conversion Conduit (Traditional IRA) into the TSP G Fund.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="53" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>6.</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Log whatever you actually transferred in the "Actual Transferred" column, even if it matches the recommendation exactly -- leaving it blank makes the sheet assume the recommendation happened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>7.</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>If the TSP G Fund is ever fully drawn down, check the Emergency Liquidity Protocol block for the next-dollar priority order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>COLOR LEGEND</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n"/>
+    </row>
+    <row r="25" ht="23" customHeight="1">
+      <c r="A25" s="5" t="n"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Pale yellow -- type your own numbers here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="23" customHeight="1">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>White (no fill) -- a formula; please leave it alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="23" customHeight="1">
+      <c r="A27" s="7" t="n"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Ice blue -- a computed summary or headline total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="23" customHeight="1">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Green (Emergency Liquidity Protocol only) -- the TSP G Fund shield is active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="38" customHeight="1">
+      <c r="A29" s="9" t="n"/>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Yellow (Emergency Liquidity Protocol only) -- the G Fund is exhausted; drawing from the cash buffer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="38" customHeight="1">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Red (Emergency Liquidity Protocol only) -- both cash shields are exhausted; the household is in an emergency-liquidation stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GLOSSARY</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="38" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>COLA</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>The federal Cost-of-Living Adjustment, applied annually to Social Security/federal retirement benefits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="38" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Hurdle Rate</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>The minimum real (inflation-adjusted) growth rate the portfolio needs to clear to be considered "on track" -- COLA layered on a fixed real-growth baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="23" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>W_t / W_q</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Total dollar outflows (withdrawals) for a given year (t) or quarter (q).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="38" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>P_track</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>The simulated target portfolio value that the household's actual wealth is measured against each year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="38" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>SRR</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Sequence-of-Returns Risk -- the risk that a downturn early in retirement forces permanent sale of depreciated assets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="38" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>TSP G Fund</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>The federal Thrift Savings Plan's government-securities fund: principal-protected, instantly liquid, and the household's operating cash vault.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="38" customHeight="1">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Safety Anchor</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>The G Fund cash buffer this engine tries to maintain, expressed as a percentage of total net worth (set on The_Refill_Engine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="38" customHeight="1">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Conduit</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>A Traditional IRA used as a pass-through for pre-tax rollovers back into the TSP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="38" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>Rollover</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>A pre-tax transfer of funds between retirement accounts (e.g. Traditional IRA to TSP) that doesn't trigger a taxable distribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="23" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Allocation Mix</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>Each account's share of total household net worth, shown on Account_Tracker.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -594,417 +1025,417 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>HOUSEHOLD VARIABLE LOG — ANNUAL HURDLE INPUTS &amp; MONTHLY TSP → CHECKING PAYMENT LOG (2026-2035)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Date / Year</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Actual Federal COLA (C_i)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Rule of Four Hurdle Baseline</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Total Annual Hurdle Rate</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Total Annual Outflows (W_t)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="11" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" s="11" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" s="11" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P2" s="11" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="Q2" s="11" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="14" t="n">
         <v>2026</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="15" t="n">
         <v>0.026</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="16">
         <f>(1+B3)*(1+C3)</f>
         <v/>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="17">
         <f>SUM(F3:Q3)</f>
         <v/>
       </c>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="7" t="n"/>
-      <c r="H3" s="7" t="n"/>
-      <c r="I3" s="7" t="n"/>
-      <c r="J3" s="7" t="n"/>
-      <c r="K3" s="7" t="n"/>
-      <c r="L3" s="7" t="n"/>
-      <c r="M3" s="7" t="n"/>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="7" t="n"/>
-      <c r="P3" s="7" t="n"/>
-      <c r="Q3" s="7" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="18" t="n"/>
+      <c r="H3" s="18" t="n"/>
+      <c r="I3" s="18" t="n"/>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="n"/>
+      <c r="L3" s="18" t="n"/>
+      <c r="M3" s="18" t="n"/>
+      <c r="N3" s="18" t="n"/>
+      <c r="O3" s="18" t="n"/>
+      <c r="P3" s="18" t="n"/>
+      <c r="Q3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="14" t="n">
         <v>2027</v>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="5" t="n">
+      <c r="B4" s="15" t="n"/>
+      <c r="C4" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="16">
         <f>(1+B4)*(1+C4)</f>
         <v/>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="17">
         <f>SUM(F4:Q4)</f>
         <v/>
       </c>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="7" t="n"/>
-      <c r="P4" s="7" t="n"/>
-      <c r="Q4" s="7" t="n"/>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="18" t="n"/>
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="18" t="n"/>
+      <c r="J4" s="18" t="n"/>
+      <c r="K4" s="18" t="n"/>
+      <c r="L4" s="18" t="n"/>
+      <c r="M4" s="18" t="n"/>
+      <c r="N4" s="18" t="n"/>
+      <c r="O4" s="18" t="n"/>
+      <c r="P4" s="18" t="n"/>
+      <c r="Q4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="14" t="n">
         <v>2028</v>
       </c>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="5" t="n">
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="16">
         <f>(1+B5)*(1+C5)</f>
         <v/>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="17">
         <f>SUM(F5:Q5)</f>
         <v/>
       </c>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="7" t="n"/>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="7" t="n"/>
-      <c r="P5" s="7" t="n"/>
-      <c r="Q5" s="7" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="18" t="n"/>
+      <c r="L5" s="18" t="n"/>
+      <c r="M5" s="18" t="n"/>
+      <c r="N5" s="18" t="n"/>
+      <c r="O5" s="18" t="n"/>
+      <c r="P5" s="18" t="n"/>
+      <c r="Q5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="14" t="n">
         <v>2029</v>
       </c>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="5" t="n">
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="16">
         <f>(1+B6)*(1+C6)</f>
         <v/>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="17">
         <f>SUM(F6:Q6)</f>
         <v/>
       </c>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
-      <c r="O6" s="7" t="n"/>
-      <c r="P6" s="7" t="n"/>
-      <c r="Q6" s="7" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="18" t="n"/>
+      <c r="J6" s="18" t="n"/>
+      <c r="K6" s="18" t="n"/>
+      <c r="L6" s="18" t="n"/>
+      <c r="M6" s="18" t="n"/>
+      <c r="N6" s="18" t="n"/>
+      <c r="O6" s="18" t="n"/>
+      <c r="P6" s="18" t="n"/>
+      <c r="Q6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="14" t="n">
         <v>2030</v>
       </c>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="5" t="n">
+      <c r="B7" s="15" t="n"/>
+      <c r="C7" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="16">
         <f>(1+B7)*(1+C7)</f>
         <v/>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="17">
         <f>SUM(F7:Q7)</f>
         <v/>
       </c>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="18" t="n"/>
+      <c r="Q7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="14" t="n">
         <v>2031</v>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="5" t="n">
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="16">
         <f>(1+B8)*(1+C8)</f>
         <v/>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="17">
         <f>SUM(F8:Q8)</f>
         <v/>
       </c>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="18" t="n"/>
+      <c r="M8" s="18" t="n"/>
+      <c r="N8" s="18" t="n"/>
+      <c r="O8" s="18" t="n"/>
+      <c r="P8" s="18" t="n"/>
+      <c r="Q8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="14" t="n">
         <v>2032</v>
       </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="5" t="n">
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="16">
         <f>(1+B9)*(1+C9)</f>
         <v/>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="17">
         <f>SUM(F9:Q9)</f>
         <v/>
       </c>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="7" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="18" t="n"/>
+      <c r="J9" s="18" t="n"/>
+      <c r="K9" s="18" t="n"/>
+      <c r="L9" s="18" t="n"/>
+      <c r="M9" s="18" t="n"/>
+      <c r="N9" s="18" t="n"/>
+      <c r="O9" s="18" t="n"/>
+      <c r="P9" s="18" t="n"/>
+      <c r="Q9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="14" t="n">
         <v>2033</v>
       </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="5" t="n">
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="16">
         <f>(1+B10)*(1+C10)</f>
         <v/>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="17">
         <f>SUM(F10:Q10)</f>
         <v/>
       </c>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
-      <c r="O10" s="7" t="n"/>
-      <c r="P10" s="7" t="n"/>
-      <c r="Q10" s="7" t="n"/>
+      <c r="F10" s="18" t="n"/>
+      <c r="G10" s="18" t="n"/>
+      <c r="H10" s="18" t="n"/>
+      <c r="I10" s="18" t="n"/>
+      <c r="J10" s="18" t="n"/>
+      <c r="K10" s="18" t="n"/>
+      <c r="L10" s="18" t="n"/>
+      <c r="M10" s="18" t="n"/>
+      <c r="N10" s="18" t="n"/>
+      <c r="O10" s="18" t="n"/>
+      <c r="P10" s="18" t="n"/>
+      <c r="Q10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="14" t="n">
         <v>2034</v>
       </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="5" t="n">
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="16">
         <f>(1+B11)*(1+C11)</f>
         <v/>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="17">
         <f>SUM(F11:Q11)</f>
         <v/>
       </c>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="7" t="n"/>
-      <c r="Q11" s="7" t="n"/>
+      <c r="F11" s="18" t="n"/>
+      <c r="G11" s="18" t="n"/>
+      <c r="H11" s="18" t="n"/>
+      <c r="I11" s="18" t="n"/>
+      <c r="J11" s="18" t="n"/>
+      <c r="K11" s="18" t="n"/>
+      <c r="L11" s="18" t="n"/>
+      <c r="M11" s="18" t="n"/>
+      <c r="N11" s="18" t="n"/>
+      <c r="O11" s="18" t="n"/>
+      <c r="P11" s="18" t="n"/>
+      <c r="Q11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="14" t="n">
         <v>2035</v>
       </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="5" t="n">
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="16">
         <f>(1+B12)*(1+C12)</f>
         <v/>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="17">
         <f>SUM(F12:Q12)</f>
         <v/>
       </c>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="7" t="n"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
-      <c r="K12" s="7" t="n"/>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="7" t="n"/>
-      <c r="Q12" s="7" t="n"/>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="18" t="n"/>
+      <c r="H12" s="18" t="n"/>
+      <c r="I12" s="18" t="n"/>
+      <c r="J12" s="18" t="n"/>
+      <c r="K12" s="18" t="n"/>
+      <c r="L12" s="18" t="n"/>
+      <c r="M12" s="18" t="n"/>
+      <c r="N12" s="18" t="n"/>
+      <c r="O12" s="18" t="n"/>
+      <c r="P12" s="18" t="n"/>
+      <c r="Q12" s="18" t="n"/>
     </row>
     <row r="13"/>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Notes: Seed 2026 COLA is set; enter 2027-2035 COLA as it is announced each fall. Log each month's actual TSP -&gt; checking payment in columns F:Q as it is set or changes -- Total Annual Outflows (E) sums automatically. If a payment amount changes mid-year, just overwrite that month's cell going forward.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Legend: pale-yellow cells are yours to type into; white cells hold formulas -- please don't overwrite them.</t>
         </is>
@@ -1018,7 +1449,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1027,192 +1458,192 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Asset Pool</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Custodian / Platform</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Live Balance</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Allocation Mix</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>Your Pre-Tax Account</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>TSP G Fund</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="18" t="n">
         <v>100000</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="16">
         <f>C2/$C$9</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Your Conversion Conduit</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Private Traditional IRA</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="18" t="n">
         <v>100000</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="16">
         <f>C3/$C$9</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Your Tax-Free Growth</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Private Roth IRA</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="18" t="n">
         <v>100000</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="16">
         <f>C4/$C$9</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Wife's Tax-Free Growth</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Spouse's Tax-Free Growth</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Private Roth IRA</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="18" t="n">
         <v>100000</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="16">
         <f>C5/$C$9</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Wife's Safe Pre-Tax Account</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Spouse's Safe Pre-Tax Account</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Current Employer 403b (Active + Reverse Rollover)</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="18" t="n">
         <v>100000</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="16">
         <f>C6/$C$9</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Wife's Conversion Conduit</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Spouse's Conversion Conduit</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Private Traditional IRA</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="18" t="n">
         <v>100000</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="16">
         <f>C7/$C$9</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Short-Term Liquidity</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Merrill Edge Cash Buffer</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="18" t="n">
         <v>100000</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="16">
         <f>C8/$C$9</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Total Household Net Worth</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="11">
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="22">
         <f>SUM(C2:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="23">
         <f>C9/C9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Note: Live Balance figures are a manually-updated snapshot -- refresh them whenever you check statements, ideally at least quarterly, so Tab 3's projections start from an accurate baseline.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Legend: pale-yellow cells are yours to type into; white cells hold formulas -- please don't overwrite them.</t>
         </is>
@@ -1223,7 +1654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1243,39 +1674,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Total Current Actual Wealth</t>
         </is>
       </c>
-      <c r="B1" s="11">
+      <c r="B1" s="22">
         <f>'Account_Tracker'!$C$9</f>
         <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Safety Anchor Target % (of Net Worth)</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n">
+      <c r="B2" s="25" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Target Safety Anchor Balance ($)</t>
         </is>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="22">
         <f>B1*B2</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Sequence-of-Returns-Risk (SRR) Shield: the Safety Anchor Target % above controls how large a G Fund cash buffer this engine tries to maintain, so equities are never forced to sell at a loss to fund living expenses. Raise or lower it to fit your risk tolerance.</t>
         </is>
@@ -1283,1297 +1714,1297 @@
     </row>
     <row r="5"/>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>THE QUARTERLY REFILL ENGINE — PRIMARY OUTPUT: RECOMMENDED TSP TOP-UP TRANSFER</t>
         </is>
       </c>
-      <c r="B6" s="1" t="n"/>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1" t="n"/>
-      <c r="H6" s="1" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Quarterly Outflow (W_q)</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Annual Performance Signal</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>G Fund Balance (Start of Qtr)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Recommended Transfer This Quarter</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Actual Transferred (Log It Here)</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>G Fund Balance (End of Qtr, Projected)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="15" t="n">
+      <c r="A8" s="26" t="n">
         <v>2026</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="28">
         <f>SUM('Variables_And_Log'!F3:H3)</f>
         <v/>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="29">
         <f>E52</f>
         <v/>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="28">
         <f>'Account_Tracker'!$C$2</f>
         <v/>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D8)),MAX(0,$B$3-E8),0)</f>
         <v/>
       </c>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="17">
+      <c r="G8" s="31" t="n"/>
+      <c r="H8" s="28">
         <f>E8-C8+IF(G8="",F8,G8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="14" t="n">
         <v>2026</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="17">
         <f>SUM('Variables_And_Log'!I3:K3)</f>
         <v/>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="32">
         <f>E52</f>
         <v/>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="17">
         <f>H8</f>
         <v/>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D9)),MAX(0,$B$3-E9),0)</f>
         <v/>
       </c>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="6">
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="17">
         <f>E9-C9+IF(G9="",F9,G9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="14" t="n">
         <v>2026</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="17">
         <f>SUM('Variables_And_Log'!L3:N3)</f>
         <v/>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="32">
         <f>E52</f>
         <v/>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="17">
         <f>H9</f>
         <v/>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D10)),MAX(0,$B$3-E10),0)</f>
         <v/>
       </c>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="6">
+      <c r="G10" s="18" t="n"/>
+      <c r="H10" s="17">
         <f>E10-C10+IF(G10="",F10,G10)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="14" t="n">
         <v>2026</v>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="17">
         <f>SUM('Variables_And_Log'!O3:Q3)</f>
         <v/>
       </c>
-      <c r="D11" s="21">
+      <c r="D11" s="32">
         <f>E52</f>
         <v/>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="17">
         <f>H10</f>
         <v/>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D11)),MAX(0,$B$3-E11),0)</f>
         <v/>
       </c>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="6">
+      <c r="G11" s="18" t="n"/>
+      <c r="H11" s="17">
         <f>E11-C11+IF(G11="",F11,G11)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="15" t="n">
+      <c r="A12" s="26" t="n">
         <v>2027</v>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="28">
         <f>SUM('Variables_And_Log'!F4:H4)</f>
         <v/>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="29">
         <f>E53</f>
         <v/>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="28">
         <f>H11</f>
         <v/>
       </c>
-      <c r="F12" s="19">
+      <c r="F12" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D12)),MAX(0,$B$3-E12),0)</f>
         <v/>
       </c>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="17">
+      <c r="G12" s="31" t="n"/>
+      <c r="H12" s="28">
         <f>E12-C12+IF(G12="",F12,G12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="14" t="n">
         <v>2027</v>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="17">
         <f>SUM('Variables_And_Log'!I4:K4)</f>
         <v/>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="32">
         <f>E53</f>
         <v/>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="17">
         <f>H12</f>
         <v/>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D13)),MAX(0,$B$3-E13),0)</f>
         <v/>
       </c>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="6">
+      <c r="G13" s="18" t="n"/>
+      <c r="H13" s="17">
         <f>E13-C13+IF(G13="",F13,G13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="14" t="n">
         <v>2027</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="17">
         <f>SUM('Variables_And_Log'!L4:N4)</f>
         <v/>
       </c>
-      <c r="D14" s="21">
+      <c r="D14" s="32">
         <f>E53</f>
         <v/>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="17">
         <f>H13</f>
         <v/>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D14)),MAX(0,$B$3-E14),0)</f>
         <v/>
       </c>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="6">
+      <c r="G14" s="18" t="n"/>
+      <c r="H14" s="17">
         <f>E14-C14+IF(G14="",F14,G14)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="14" t="n">
         <v>2027</v>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="17">
         <f>SUM('Variables_And_Log'!O4:Q4)</f>
         <v/>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="32">
         <f>E53</f>
         <v/>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="17">
         <f>H14</f>
         <v/>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D15)),MAX(0,$B$3-E15),0)</f>
         <v/>
       </c>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="6">
+      <c r="G15" s="18" t="n"/>
+      <c r="H15" s="17">
         <f>E15-C15+IF(G15="",F15,G15)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="15" t="n">
+      <c r="A16" s="26" t="n">
         <v>2028</v>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="28">
         <f>SUM('Variables_And_Log'!F5:H5)</f>
         <v/>
       </c>
-      <c r="D16" s="18">
+      <c r="D16" s="29">
         <f>E54</f>
         <v/>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="28">
         <f>H15</f>
         <v/>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D16)),MAX(0,$B$3-E16),0)</f>
         <v/>
       </c>
-      <c r="G16" s="20" t="n"/>
-      <c r="H16" s="17">
+      <c r="G16" s="31" t="n"/>
+      <c r="H16" s="28">
         <f>E16-C16+IF(G16="",F16,G16)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="14" t="n">
         <v>2028</v>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="17">
         <f>SUM('Variables_And_Log'!I5:K5)</f>
         <v/>
       </c>
-      <c r="D17" s="21">
+      <c r="D17" s="32">
         <f>E54</f>
         <v/>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="17">
         <f>H16</f>
         <v/>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D17)),MAX(0,$B$3-E17),0)</f>
         <v/>
       </c>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="6">
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="17">
         <f>E17-C17+IF(G17="",F17,G17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="14" t="n">
         <v>2028</v>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="17">
         <f>SUM('Variables_And_Log'!L5:N5)</f>
         <v/>
       </c>
-      <c r="D18" s="21">
+      <c r="D18" s="32">
         <f>E54</f>
         <v/>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="17">
         <f>H17</f>
         <v/>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D18)),MAX(0,$B$3-E18),0)</f>
         <v/>
       </c>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="6">
+      <c r="G18" s="18" t="n"/>
+      <c r="H18" s="17">
         <f>E18-C18+IF(G18="",F18,G18)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="14" t="n">
         <v>2028</v>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="17">
         <f>SUM('Variables_And_Log'!O5:Q5)</f>
         <v/>
       </c>
-      <c r="D19" s="21">
+      <c r="D19" s="32">
         <f>E54</f>
         <v/>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="17">
         <f>H18</f>
         <v/>
       </c>
-      <c r="F19" s="11">
+      <c r="F19" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D19)),MAX(0,$B$3-E19),0)</f>
         <v/>
       </c>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="6">
+      <c r="G19" s="18" t="n"/>
+      <c r="H19" s="17">
         <f>E19-C19+IF(G19="",F19,G19)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="15" t="n">
+      <c r="A20" s="26" t="n">
         <v>2029</v>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="28">
         <f>SUM('Variables_And_Log'!F6:H6)</f>
         <v/>
       </c>
-      <c r="D20" s="18">
+      <c r="D20" s="29">
         <f>E55</f>
         <v/>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="28">
         <f>H19</f>
         <v/>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D20)),MAX(0,$B$3-E20),0)</f>
         <v/>
       </c>
-      <c r="G20" s="20" t="n"/>
-      <c r="H20" s="17">
+      <c r="G20" s="31" t="n"/>
+      <c r="H20" s="28">
         <f>E20-C20+IF(G20="",F20,G20)</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="14" t="n">
         <v>2029</v>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="17">
         <f>SUM('Variables_And_Log'!I6:K6)</f>
         <v/>
       </c>
-      <c r="D21" s="21">
+      <c r="D21" s="32">
         <f>E55</f>
         <v/>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="17">
         <f>H20</f>
         <v/>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D21)),MAX(0,$B$3-E21),0)</f>
         <v/>
       </c>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="6">
+      <c r="G21" s="18" t="n"/>
+      <c r="H21" s="17">
         <f>E21-C21+IF(G21="",F21,G21)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="14" t="n">
         <v>2029</v>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="17">
         <f>SUM('Variables_And_Log'!L6:N6)</f>
         <v/>
       </c>
-      <c r="D22" s="21">
+      <c r="D22" s="32">
         <f>E55</f>
         <v/>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="17">
         <f>H21</f>
         <v/>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D22)),MAX(0,$B$3-E22),0)</f>
         <v/>
       </c>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="6">
+      <c r="G22" s="18" t="n"/>
+      <c r="H22" s="17">
         <f>E22-C22+IF(G22="",F22,G22)</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="14" t="n">
         <v>2029</v>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="17">
         <f>SUM('Variables_And_Log'!O6:Q6)</f>
         <v/>
       </c>
-      <c r="D23" s="21">
+      <c r="D23" s="32">
         <f>E55</f>
         <v/>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="17">
         <f>H22</f>
         <v/>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D23)),MAX(0,$B$3-E23),0)</f>
         <v/>
       </c>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="6">
+      <c r="G23" s="18" t="n"/>
+      <c r="H23" s="17">
         <f>E23-C23+IF(G23="",F23,G23)</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="15" t="n">
+      <c r="A24" s="26" t="n">
         <v>2030</v>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="28">
         <f>SUM('Variables_And_Log'!F7:H7)</f>
         <v/>
       </c>
-      <c r="D24" s="18">
+      <c r="D24" s="29">
         <f>E56</f>
         <v/>
       </c>
-      <c r="E24" s="17">
+      <c r="E24" s="28">
         <f>H23</f>
         <v/>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D24)),MAX(0,$B$3-E24),0)</f>
         <v/>
       </c>
-      <c r="G24" s="20" t="n"/>
-      <c r="H24" s="17">
+      <c r="G24" s="31" t="n"/>
+      <c r="H24" s="28">
         <f>E24-C24+IF(G24="",F24,G24)</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="14" t="n">
         <v>2030</v>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="17">
         <f>SUM('Variables_And_Log'!I7:K7)</f>
         <v/>
       </c>
-      <c r="D25" s="21">
+      <c r="D25" s="32">
         <f>E56</f>
         <v/>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="17">
         <f>H24</f>
         <v/>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D25)),MAX(0,$B$3-E25),0)</f>
         <v/>
       </c>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="6">
+      <c r="G25" s="18" t="n"/>
+      <c r="H25" s="17">
         <f>E25-C25+IF(G25="",F25,G25)</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="3" t="n">
+      <c r="A26" s="14" t="n">
         <v>2030</v>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="17">
         <f>SUM('Variables_And_Log'!L7:N7)</f>
         <v/>
       </c>
-      <c r="D26" s="21">
+      <c r="D26" s="32">
         <f>E56</f>
         <v/>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="17">
         <f>H25</f>
         <v/>
       </c>
-      <c r="F26" s="11">
+      <c r="F26" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D26)),MAX(0,$B$3-E26),0)</f>
         <v/>
       </c>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="6">
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="17">
         <f>E26-C26+IF(G26="",F26,G26)</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="3" t="n">
+      <c r="A27" s="14" t="n">
         <v>2030</v>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="17">
         <f>SUM('Variables_And_Log'!O7:Q7)</f>
         <v/>
       </c>
-      <c r="D27" s="21">
+      <c r="D27" s="32">
         <f>E56</f>
         <v/>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="17">
         <f>H26</f>
         <v/>
       </c>
-      <c r="F27" s="11">
+      <c r="F27" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D27)),MAX(0,$B$3-E27),0)</f>
         <v/>
       </c>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="6">
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="17">
         <f>E27-C27+IF(G27="",F27,G27)</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="15" t="n">
+      <c r="A28" s="26" t="n">
         <v>2031</v>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C28" s="17">
+      <c r="C28" s="28">
         <f>SUM('Variables_And_Log'!F8:H8)</f>
         <v/>
       </c>
-      <c r="D28" s="18">
+      <c r="D28" s="29">
         <f>E57</f>
         <v/>
       </c>
-      <c r="E28" s="17">
+      <c r="E28" s="28">
         <f>H27</f>
         <v/>
       </c>
-      <c r="F28" s="19">
+      <c r="F28" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D28)),MAX(0,$B$3-E28),0)</f>
         <v/>
       </c>
-      <c r="G28" s="20" t="n"/>
-      <c r="H28" s="17">
+      <c r="G28" s="31" t="n"/>
+      <c r="H28" s="28">
         <f>E28-C28+IF(G28="",F28,G28)</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="3" t="n">
+      <c r="A29" s="14" t="n">
         <v>2031</v>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="17">
         <f>SUM('Variables_And_Log'!I8:K8)</f>
         <v/>
       </c>
-      <c r="D29" s="21">
+      <c r="D29" s="32">
         <f>E57</f>
         <v/>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="17">
         <f>H28</f>
         <v/>
       </c>
-      <c r="F29" s="11">
+      <c r="F29" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D29)),MAX(0,$B$3-E29),0)</f>
         <v/>
       </c>
-      <c r="G29" s="7" t="n"/>
-      <c r="H29" s="6">
+      <c r="G29" s="18" t="n"/>
+      <c r="H29" s="17">
         <f>E29-C29+IF(G29="",F29,G29)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="3" t="n">
+      <c r="A30" s="14" t="n">
         <v>2031</v>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="17">
         <f>SUM('Variables_And_Log'!L8:N8)</f>
         <v/>
       </c>
-      <c r="D30" s="21">
+      <c r="D30" s="32">
         <f>E57</f>
         <v/>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="17">
         <f>H29</f>
         <v/>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D30)),MAX(0,$B$3-E30),0)</f>
         <v/>
       </c>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="6">
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="17">
         <f>E30-C30+IF(G30="",F30,G30)</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="3" t="n">
+      <c r="A31" s="14" t="n">
         <v>2031</v>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="17">
         <f>SUM('Variables_And_Log'!O8:Q8)</f>
         <v/>
       </c>
-      <c r="D31" s="21">
+      <c r="D31" s="32">
         <f>E57</f>
         <v/>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="17">
         <f>H30</f>
         <v/>
       </c>
-      <c r="F31" s="11">
+      <c r="F31" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D31)),MAX(0,$B$3-E31),0)</f>
         <v/>
       </c>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="6">
+      <c r="G31" s="18" t="n"/>
+      <c r="H31" s="17">
         <f>E31-C31+IF(G31="",F31,G31)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="15" t="n">
+      <c r="A32" s="26" t="n">
         <v>2032</v>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B32" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C32" s="17">
+      <c r="C32" s="28">
         <f>SUM('Variables_And_Log'!F9:H9)</f>
         <v/>
       </c>
-      <c r="D32" s="18">
+      <c r="D32" s="29">
         <f>E58</f>
         <v/>
       </c>
-      <c r="E32" s="17">
+      <c r="E32" s="28">
         <f>H31</f>
         <v/>
       </c>
-      <c r="F32" s="19">
+      <c r="F32" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D32)),MAX(0,$B$3-E32),0)</f>
         <v/>
       </c>
-      <c r="G32" s="20" t="n"/>
-      <c r="H32" s="17">
+      <c r="G32" s="31" t="n"/>
+      <c r="H32" s="28">
         <f>E32-C32+IF(G32="",F32,G32)</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="3" t="n">
+      <c r="A33" s="14" t="n">
         <v>2032</v>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C33" s="6">
+      <c r="C33" s="17">
         <f>SUM('Variables_And_Log'!I9:K9)</f>
         <v/>
       </c>
-      <c r="D33" s="21">
+      <c r="D33" s="32">
         <f>E58</f>
         <v/>
       </c>
-      <c r="E33" s="6">
+      <c r="E33" s="17">
         <f>H32</f>
         <v/>
       </c>
-      <c r="F33" s="11">
+      <c r="F33" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D33)),MAX(0,$B$3-E33),0)</f>
         <v/>
       </c>
-      <c r="G33" s="7" t="n"/>
-      <c r="H33" s="6">
+      <c r="G33" s="18" t="n"/>
+      <c r="H33" s="17">
         <f>E33-C33+IF(G33="",F33,G33)</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="3" t="n">
+      <c r="A34" s="14" t="n">
         <v>2032</v>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C34" s="6">
+      <c r="C34" s="17">
         <f>SUM('Variables_And_Log'!L9:N9)</f>
         <v/>
       </c>
-      <c r="D34" s="21">
+      <c r="D34" s="32">
         <f>E58</f>
         <v/>
       </c>
-      <c r="E34" s="6">
+      <c r="E34" s="17">
         <f>H33</f>
         <v/>
       </c>
-      <c r="F34" s="11">
+      <c r="F34" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D34)),MAX(0,$B$3-E34),0)</f>
         <v/>
       </c>
-      <c r="G34" s="7" t="n"/>
-      <c r="H34" s="6">
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="17">
         <f>E34-C34+IF(G34="",F34,G34)</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="3" t="n">
+      <c r="A35" s="14" t="n">
         <v>2032</v>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C35" s="6">
+      <c r="C35" s="17">
         <f>SUM('Variables_And_Log'!O9:Q9)</f>
         <v/>
       </c>
-      <c r="D35" s="21">
+      <c r="D35" s="32">
         <f>E58</f>
         <v/>
       </c>
-      <c r="E35" s="6">
+      <c r="E35" s="17">
         <f>H34</f>
         <v/>
       </c>
-      <c r="F35" s="11">
+      <c r="F35" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D35)),MAX(0,$B$3-E35),0)</f>
         <v/>
       </c>
-      <c r="G35" s="7" t="n"/>
-      <c r="H35" s="6">
+      <c r="G35" s="18" t="n"/>
+      <c r="H35" s="17">
         <f>E35-C35+IF(G35="",F35,G35)</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="15" t="n">
+      <c r="A36" s="26" t="n">
         <v>2033</v>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B36" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C36" s="17">
+      <c r="C36" s="28">
         <f>SUM('Variables_And_Log'!F10:H10)</f>
         <v/>
       </c>
-      <c r="D36" s="18">
+      <c r="D36" s="29">
         <f>E59</f>
         <v/>
       </c>
-      <c r="E36" s="17">
+      <c r="E36" s="28">
         <f>H35</f>
         <v/>
       </c>
-      <c r="F36" s="19">
+      <c r="F36" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D36)),MAX(0,$B$3-E36),0)</f>
         <v/>
       </c>
-      <c r="G36" s="20" t="n"/>
-      <c r="H36" s="17">
+      <c r="G36" s="31" t="n"/>
+      <c r="H36" s="28">
         <f>E36-C36+IF(G36="",F36,G36)</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="3" t="n">
+      <c r="A37" s="14" t="n">
         <v>2033</v>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C37" s="6">
+      <c r="C37" s="17">
         <f>SUM('Variables_And_Log'!I10:K10)</f>
         <v/>
       </c>
-      <c r="D37" s="21">
+      <c r="D37" s="32">
         <f>E59</f>
         <v/>
       </c>
-      <c r="E37" s="6">
+      <c r="E37" s="17">
         <f>H36</f>
         <v/>
       </c>
-      <c r="F37" s="11">
+      <c r="F37" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D37)),MAX(0,$B$3-E37),0)</f>
         <v/>
       </c>
-      <c r="G37" s="7" t="n"/>
-      <c r="H37" s="6">
+      <c r="G37" s="18" t="n"/>
+      <c r="H37" s="17">
         <f>E37-C37+IF(G37="",F37,G37)</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="3" t="n">
+      <c r="A38" s="14" t="n">
         <v>2033</v>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B38" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C38" s="6">
+      <c r="C38" s="17">
         <f>SUM('Variables_And_Log'!L10:N10)</f>
         <v/>
       </c>
-      <c r="D38" s="21">
+      <c r="D38" s="32">
         <f>E59</f>
         <v/>
       </c>
-      <c r="E38" s="6">
+      <c r="E38" s="17">
         <f>H37</f>
         <v/>
       </c>
-      <c r="F38" s="11">
+      <c r="F38" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D38)),MAX(0,$B$3-E38),0)</f>
         <v/>
       </c>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="6">
+      <c r="G38" s="18" t="n"/>
+      <c r="H38" s="17">
         <f>E38-C38+IF(G38="",F38,G38)</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="3" t="n">
+      <c r="A39" s="14" t="n">
         <v>2033</v>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B39" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C39" s="6">
+      <c r="C39" s="17">
         <f>SUM('Variables_And_Log'!O10:Q10)</f>
         <v/>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="32">
         <f>E59</f>
         <v/>
       </c>
-      <c r="E39" s="6">
+      <c r="E39" s="17">
         <f>H38</f>
         <v/>
       </c>
-      <c r="F39" s="11">
+      <c r="F39" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D39)),MAX(0,$B$3-E39),0)</f>
         <v/>
       </c>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="6">
+      <c r="G39" s="18" t="n"/>
+      <c r="H39" s="17">
         <f>E39-C39+IF(G39="",F39,G39)</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="15" t="n">
+      <c r="A40" s="26" t="n">
         <v>2034</v>
       </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="B40" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C40" s="17">
+      <c r="C40" s="28">
         <f>SUM('Variables_And_Log'!F11:H11)</f>
         <v/>
       </c>
-      <c r="D40" s="18">
+      <c r="D40" s="29">
         <f>E60</f>
         <v/>
       </c>
-      <c r="E40" s="17">
+      <c r="E40" s="28">
         <f>H39</f>
         <v/>
       </c>
-      <c r="F40" s="19">
+      <c r="F40" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D40)),MAX(0,$B$3-E40),0)</f>
         <v/>
       </c>
-      <c r="G40" s="20" t="n"/>
-      <c r="H40" s="17">
+      <c r="G40" s="31" t="n"/>
+      <c r="H40" s="28">
         <f>E40-C40+IF(G40="",F40,G40)</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="3" t="n">
+      <c r="A41" s="14" t="n">
         <v>2034</v>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B41" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C41" s="6">
+      <c r="C41" s="17">
         <f>SUM('Variables_And_Log'!I11:K11)</f>
         <v/>
       </c>
-      <c r="D41" s="21">
+      <c r="D41" s="32">
         <f>E60</f>
         <v/>
       </c>
-      <c r="E41" s="6">
+      <c r="E41" s="17">
         <f>H40</f>
         <v/>
       </c>
-      <c r="F41" s="11">
+      <c r="F41" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D41)),MAX(0,$B$3-E41),0)</f>
         <v/>
       </c>
-      <c r="G41" s="7" t="n"/>
-      <c r="H41" s="6">
+      <c r="G41" s="18" t="n"/>
+      <c r="H41" s="17">
         <f>E41-C41+IF(G41="",F41,G41)</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="3" t="n">
+      <c r="A42" s="14" t="n">
         <v>2034</v>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B42" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C42" s="6">
+      <c r="C42" s="17">
         <f>SUM('Variables_And_Log'!L11:N11)</f>
         <v/>
       </c>
-      <c r="D42" s="21">
+      <c r="D42" s="32">
         <f>E60</f>
         <v/>
       </c>
-      <c r="E42" s="6">
+      <c r="E42" s="17">
         <f>H41</f>
         <v/>
       </c>
-      <c r="F42" s="11">
+      <c r="F42" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D42)),MAX(0,$B$3-E42),0)</f>
         <v/>
       </c>
-      <c r="G42" s="7" t="n"/>
-      <c r="H42" s="6">
+      <c r="G42" s="18" t="n"/>
+      <c r="H42" s="17">
         <f>E42-C42+IF(G42="",F42,G42)</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1">
-      <c r="A43" s="3" t="n">
+      <c r="A43" s="14" t="n">
         <v>2034</v>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B43" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C43" s="6">
+      <c r="C43" s="17">
         <f>SUM('Variables_And_Log'!O11:Q11)</f>
         <v/>
       </c>
-      <c r="D43" s="21">
+      <c r="D43" s="32">
         <f>E60</f>
         <v/>
       </c>
-      <c r="E43" s="6">
+      <c r="E43" s="17">
         <f>H42</f>
         <v/>
       </c>
-      <c r="F43" s="11">
+      <c r="F43" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D43)),MAX(0,$B$3-E43),0)</f>
         <v/>
       </c>
-      <c r="G43" s="7" t="n"/>
-      <c r="H43" s="6">
+      <c r="G43" s="18" t="n"/>
+      <c r="H43" s="17">
         <f>E43-C43+IF(G43="",F43,G43)</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="15" t="n">
+      <c r="A44" s="26" t="n">
         <v>2035</v>
       </c>
-      <c r="B44" s="16" t="inlineStr">
+      <c r="B44" s="27" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C44" s="17">
+      <c r="C44" s="28">
         <f>SUM('Variables_And_Log'!F12:H12)</f>
         <v/>
       </c>
-      <c r="D44" s="18">
+      <c r="D44" s="29">
         <f>E61</f>
         <v/>
       </c>
-      <c r="E44" s="17">
+      <c r="E44" s="28">
         <f>H43</f>
         <v/>
       </c>
-      <c r="F44" s="19">
+      <c r="F44" s="30">
         <f>IF(ISNUMBER(SEARCH("GOOD",D44)),MAX(0,$B$3-E44),0)</f>
         <v/>
       </c>
-      <c r="G44" s="20" t="n"/>
-      <c r="H44" s="17">
+      <c r="G44" s="31" t="n"/>
+      <c r="H44" s="28">
         <f>E44-C44+IF(G44="",F44,G44)</f>
         <v/>
       </c>
     </row>
     <row r="45" ht="28" customHeight="1">
-      <c r="A45" s="3" t="n">
+      <c r="A45" s="14" t="n">
         <v>2035</v>
       </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B45" s="20" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C45" s="6">
+      <c r="C45" s="17">
         <f>SUM('Variables_And_Log'!I12:K12)</f>
         <v/>
       </c>
-      <c r="D45" s="21">
+      <c r="D45" s="32">
         <f>E61</f>
         <v/>
       </c>
-      <c r="E45" s="6">
+      <c r="E45" s="17">
         <f>H44</f>
         <v/>
       </c>
-      <c r="F45" s="11">
+      <c r="F45" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D45)),MAX(0,$B$3-E45),0)</f>
         <v/>
       </c>
-      <c r="G45" s="7" t="n"/>
-      <c r="H45" s="6">
+      <c r="G45" s="18" t="n"/>
+      <c r="H45" s="17">
         <f>E45-C45+IF(G45="",F45,G45)</f>
         <v/>
       </c>
     </row>
     <row r="46" ht="28" customHeight="1">
-      <c r="A46" s="3" t="n">
+      <c r="A46" s="14" t="n">
         <v>2035</v>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B46" s="20" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C46" s="6">
+      <c r="C46" s="17">
         <f>SUM('Variables_And_Log'!L12:N12)</f>
         <v/>
       </c>
-      <c r="D46" s="21">
+      <c r="D46" s="32">
         <f>E61</f>
         <v/>
       </c>
-      <c r="E46" s="6">
+      <c r="E46" s="17">
         <f>H45</f>
         <v/>
       </c>
-      <c r="F46" s="11">
+      <c r="F46" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D46)),MAX(0,$B$3-E46),0)</f>
         <v/>
       </c>
-      <c r="G46" s="7" t="n"/>
-      <c r="H46" s="6">
+      <c r="G46" s="18" t="n"/>
+      <c r="H46" s="17">
         <f>E46-C46+IF(G46="",F46,G46)</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1">
-      <c r="A47" s="3" t="n">
+      <c r="A47" s="14" t="n">
         <v>2035</v>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B47" s="20" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C47" s="6">
+      <c r="C47" s="17">
         <f>SUM('Variables_And_Log'!O12:Q12)</f>
         <v/>
       </c>
-      <c r="D47" s="21">
+      <c r="D47" s="32">
         <f>E61</f>
         <v/>
       </c>
-      <c r="E47" s="6">
+      <c r="E47" s="17">
         <f>H46</f>
         <v/>
       </c>
-      <c r="F47" s="11">
+      <c r="F47" s="22">
         <f>IF(ISNUMBER(SEARCH("GOOD",D47)),MAX(0,$B$3-E47),0)</f>
         <v/>
       </c>
-      <c r="G47" s="7" t="n"/>
-      <c r="H47" s="6">
+      <c r="G47" s="18" t="n"/>
+      <c r="H47" s="17">
         <f>E47-C47+IF(G47="",F47,G47)</f>
         <v/>
       </c>
@@ -2581,296 +3012,296 @@
     <row r="48"/>
     <row r="49"/>
     <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="1" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>ANNUAL SRR HURDLE MODEL — STRATEGIC PACING CHECK (GATES THE QUARTERLY REFILL ABOVE)</t>
         </is>
       </c>
-      <c r="B50" s="1" t="n"/>
-      <c r="C50" s="1" t="n"/>
-      <c r="D50" s="1" t="n"/>
-      <c r="E50" s="1" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
     </row>
     <row r="51" ht="32" customHeight="1">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" s="11" t="inlineStr">
         <is>
           <t>Total Annual Hurdle Rate</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>Annual Outflows (W_t)</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" s="11" t="inlineStr">
         <is>
           <t>Simulated Target Portfolio (P_track)</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E51" s="11" t="inlineStr">
         <is>
           <t>Performance Logic Trigger</t>
         </is>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1">
-      <c r="A52" s="3" t="n">
+      <c r="A52" s="14" t="n">
         <v>2026</v>
       </c>
-      <c r="B52" s="5">
+      <c r="B52" s="16">
         <f>'Variables_And_Log'!D3</f>
         <v/>
       </c>
-      <c r="C52" s="6">
+      <c r="C52" s="17">
         <f>'Variables_And_Log'!E3</f>
         <v/>
       </c>
-      <c r="D52" s="6">
+      <c r="D52" s="17">
         <f>ROUND(($B$1*B52)-C52,2)</f>
         <v/>
       </c>
-      <c r="E52" s="21">
+      <c r="E52" s="32">
         <f>IF(B$1&gt;=D52,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="3" t="n">
+      <c r="A53" s="14" t="n">
         <v>2027</v>
       </c>
-      <c r="B53" s="5">
+      <c r="B53" s="16">
         <f>'Variables_And_Log'!D4</f>
         <v/>
       </c>
-      <c r="C53" s="6">
+      <c r="C53" s="17">
         <f>'Variables_And_Log'!E4</f>
         <v/>
       </c>
-      <c r="D53" s="6">
+      <c r="D53" s="17">
         <f>ROUND((D52*B53)-C53,2)</f>
         <v/>
       </c>
-      <c r="E53" s="21">
+      <c r="E53" s="32">
         <f>IF(B$1&gt;=D53,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="3" t="n">
+      <c r="A54" s="14" t="n">
         <v>2028</v>
       </c>
-      <c r="B54" s="5">
+      <c r="B54" s="16">
         <f>'Variables_And_Log'!D5</f>
         <v/>
       </c>
-      <c r="C54" s="6">
+      <c r="C54" s="17">
         <f>'Variables_And_Log'!E5</f>
         <v/>
       </c>
-      <c r="D54" s="6">
+      <c r="D54" s="17">
         <f>ROUND((D53*B54)-C54,2)</f>
         <v/>
       </c>
-      <c r="E54" s="21">
+      <c r="E54" s="32">
         <f>IF(B$1&gt;=D54,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="3" t="n">
+      <c r="A55" s="14" t="n">
         <v>2029</v>
       </c>
-      <c r="B55" s="5">
+      <c r="B55" s="16">
         <f>'Variables_And_Log'!D6</f>
         <v/>
       </c>
-      <c r="C55" s="6">
+      <c r="C55" s="17">
         <f>'Variables_And_Log'!E6</f>
         <v/>
       </c>
-      <c r="D55" s="6">
+      <c r="D55" s="17">
         <f>ROUND((D54*B55)-C55,2)</f>
         <v/>
       </c>
-      <c r="E55" s="21">
+      <c r="E55" s="32">
         <f>IF(B$1&gt;=D55,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="3" t="n">
+      <c r="A56" s="14" t="n">
         <v>2030</v>
       </c>
-      <c r="B56" s="5">
+      <c r="B56" s="16">
         <f>'Variables_And_Log'!D7</f>
         <v/>
       </c>
-      <c r="C56" s="6">
+      <c r="C56" s="17">
         <f>'Variables_And_Log'!E7</f>
         <v/>
       </c>
-      <c r="D56" s="6">
+      <c r="D56" s="17">
         <f>ROUND((D55*B56)-C56,2)</f>
         <v/>
       </c>
-      <c r="E56" s="21">
+      <c r="E56" s="32">
         <f>IF(B$1&gt;=D56,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="57" ht="28" customHeight="1">
-      <c r="A57" s="3" t="n">
+      <c r="A57" s="14" t="n">
         <v>2031</v>
       </c>
-      <c r="B57" s="5">
+      <c r="B57" s="16">
         <f>'Variables_And_Log'!D8</f>
         <v/>
       </c>
-      <c r="C57" s="6">
+      <c r="C57" s="17">
         <f>'Variables_And_Log'!E8</f>
         <v/>
       </c>
-      <c r="D57" s="6">
+      <c r="D57" s="17">
         <f>ROUND((D56*B57)-C57,2)</f>
         <v/>
       </c>
-      <c r="E57" s="21">
+      <c r="E57" s="32">
         <f>IF(B$1&gt;=D57,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="3" t="n">
+      <c r="A58" s="14" t="n">
         <v>2032</v>
       </c>
-      <c r="B58" s="5">
+      <c r="B58" s="16">
         <f>'Variables_And_Log'!D9</f>
         <v/>
       </c>
-      <c r="C58" s="6">
+      <c r="C58" s="17">
         <f>'Variables_And_Log'!E9</f>
         <v/>
       </c>
-      <c r="D58" s="6">
+      <c r="D58" s="17">
         <f>ROUND((D57*B58)-C58,2)</f>
         <v/>
       </c>
-      <c r="E58" s="21">
+      <c r="E58" s="32">
         <f>IF(B$1&gt;=D58,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="3" t="n">
+      <c r="A59" s="14" t="n">
         <v>2033</v>
       </c>
-      <c r="B59" s="5">
+      <c r="B59" s="16">
         <f>'Variables_And_Log'!D10</f>
         <v/>
       </c>
-      <c r="C59" s="6">
+      <c r="C59" s="17">
         <f>'Variables_And_Log'!E10</f>
         <v/>
       </c>
-      <c r="D59" s="6">
+      <c r="D59" s="17">
         <f>ROUND((D58*B59)-C59,2)</f>
         <v/>
       </c>
-      <c r="E59" s="21">
+      <c r="E59" s="32">
         <f>IF(B$1&gt;=D59,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="3" t="n">
+      <c r="A60" s="14" t="n">
         <v>2034</v>
       </c>
-      <c r="B60" s="5">
+      <c r="B60" s="16">
         <f>'Variables_And_Log'!D11</f>
         <v/>
       </c>
-      <c r="C60" s="6">
+      <c r="C60" s="17">
         <f>'Variables_And_Log'!E11</f>
         <v/>
       </c>
-      <c r="D60" s="6">
+      <c r="D60" s="17">
         <f>ROUND((D59*B60)-C60,2)</f>
         <v/>
       </c>
-      <c r="E60" s="21">
+      <c r="E60" s="32">
         <f>IF(B$1&gt;=D60,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="61" ht="28" customHeight="1">
-      <c r="A61" s="3" t="n">
+      <c r="A61" s="14" t="n">
         <v>2035</v>
       </c>
-      <c r="B61" s="5">
+      <c r="B61" s="16">
         <f>'Variables_And_Log'!D12</f>
         <v/>
       </c>
-      <c r="C61" s="6">
+      <c r="C61" s="17">
         <f>'Variables_And_Log'!E12</f>
         <v/>
       </c>
-      <c r="D61" s="6">
+      <c r="D61" s="17">
         <f>ROUND((D60*B61)-C61,2)</f>
         <v/>
       </c>
-      <c r="E61" s="21">
+      <c r="E61" s="32">
         <f>IF(B$1&gt;=D61,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
     </row>
     <row r="62"/>
     <row r="63">
-      <c r="A63" s="1" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>EXTRA CAPACITY INDICATORS</t>
         </is>
       </c>
-      <c r="B63" s="1" t="n"/>
-      <c r="C63" s="1" t="n"/>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="2" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="13" t="inlineStr">
+      <c r="A64" s="24" t="inlineStr">
         <is>
           <t>Your Pre-Tax Rollover Conduit Capacity</t>
         </is>
       </c>
-      <c r="B64" s="6">
+      <c r="B64" s="17">
         <f>'Account_Tracker'!$C$3</f>
         <v/>
       </c>
-      <c r="C64" s="10">
+      <c r="C64" s="21">
         <f>IF(B64&gt;0,"Conduit Open","Conduit Closed")</f>
         <v/>
       </c>
     </row>
     <row r="65"/>
     <row r="66">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="A66" s="24" t="inlineStr">
         <is>
           <t>TSP Cash Buffer Runway (Months)</t>
         </is>
       </c>
-      <c r="B66" s="22">
+      <c r="B66" s="33">
         <f>IFERROR('Account_Tracker'!$C$2/AVERAGE('Variables_And_Log'!$F$3:$Q$3),"Log Monthly Payments to Calculate")</f>
         <v/>
       </c>
-      <c r="C66" s="10">
+      <c r="C66" s="21">
         <f>IF(ISNUMBER(B66),IF(B66&gt;36,"Safe: 3+ Year Volatility Shield","Caution: Shield Shrinking"),"Awaiting Payment Data")</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="A67" s="19" t="inlineStr">
         <is>
           <t>(Runway uses the average of whichever 2026 monthly TSP payments you've logged so far.)</t>
         </is>
@@ -2878,45 +3309,45 @@
     </row>
     <row r="68"/>
     <row r="69">
-      <c r="A69" s="1" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>EMERGENCY LIQUIDITY PROTOCOL — NEXT-DOLLAR PRIORITY ENGINE</t>
         </is>
       </c>
-      <c r="B69" s="1" t="n"/>
-      <c r="C69" s="1" t="n"/>
-      <c r="D69" s="1" t="n"/>
-      <c r="E69" s="1" t="n"/>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="n"/>
     </row>
     <row r="70" ht="60" customHeight="1">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="A70" s="24" t="inlineStr">
         <is>
           <t>Next-Dollar Liquidity Priority</t>
         </is>
       </c>
-      <c r="B70" s="23">
-        <f>IF('Account_Tracker'!$C$2&gt;0,"🛡️ SHIELD ACTIVE: Continue automated monthly draws directly from the TSP G Fund. Your equity engines are fully insulated from sequence-of-returns risk.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8&gt;0),"⚠️ SHIELD BROKEN: TSP G Fund is exhausted. IMMEDIATELY divert monthly checking draws to your Merrill Edge Cash Buffer. This buys next-day liquidity via Bank of America without forced retirement asset sales.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8=0,'Account_Tracker'!$C$6&gt;0),"🚨 EMERGENCY LIQUIDATION - STAGE 1: G Fund and Cash Buffers are exhausted. Turn on monthly distributions from Wife's Current Employer 403b. Her pre-tax employer plan qualifies for the Maryland Pension Exclusion at age 65, making it more tax-efficient than touching your private traditional IRA.","💥 NUCLEAR PROTOCOL - STAGE 2: Absolute liquidity crisis. You are forced to break all shields. Begin selling shares of the 2065 Target Date Funds within your Private Traditional IRAs to fund monthly expenses. Maximize tax withholding at the time of distribution to shield your remaining capital from underpayment penalties.")))</f>
-        <v/>
-      </c>
-      <c r="C70" s="24" t="n"/>
-      <c r="D70" s="24" t="n"/>
-      <c r="E70" s="24" t="n"/>
+      <c r="B70" s="34">
+        <f>IF('Account_Tracker'!$C$2&gt;0,"🛡️ SHIELD ACTIVE: Continue automated monthly draws directly from the TSP G Fund. Your equity engines are fully insulated from sequence-of-returns risk.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8&gt;0),"⚠️ SHIELD BROKEN: TSP G Fund is exhausted. IMMEDIATELY divert monthly checking draws to your Merrill Edge Cash Buffer. This buys next-day liquidity via Bank of America without forced retirement asset sales.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8=0,'Account_Tracker'!$C$6&gt;0),"🚨 EMERGENCY LIQUIDATION - STAGE 1: G Fund and Cash Buffers are exhausted. Turn on monthly distributions from Spouse's Current Employer 403b. Their pre-tax employer plan qualifies for the Maryland Pension Exclusion at age 65, making it more tax-efficient than touching your private traditional IRA.","💥 NUCLEAR PROTOCOL - STAGE 2: Absolute liquidity crisis. You are forced to break all shields. Begin selling shares of the 2065 Target Date Funds within your Private Traditional IRAs to fund monthly expenses. Maximize tax withholding at the time of distribution to shield your remaining capital from underpayment penalties.")))</f>
+        <v/>
+      </c>
+      <c r="C70" s="6" t="n"/>
+      <c r="D70" s="6" t="n"/>
+      <c r="E70" s="6" t="n"/>
     </row>
     <row r="71" ht="20" customHeight="1">
-      <c r="B71" s="24" t="n"/>
-      <c r="C71" s="24" t="n"/>
-      <c r="D71" s="24" t="n"/>
-      <c r="E71" s="24" t="n"/>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="6" t="n"/>
+      <c r="D71" s="6" t="n"/>
+      <c r="E71" s="6" t="n"/>
     </row>
     <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="24" t="n"/>
-      <c r="C72" s="24" t="n"/>
-      <c r="D72" s="24" t="n"/>
-      <c r="E72" s="24" t="n"/>
+      <c r="B72" s="6" t="n"/>
+      <c r="C72" s="6" t="n"/>
+      <c r="D72" s="6" t="n"/>
+      <c r="E72" s="6" t="n"/>
     </row>
     <row r="73"/>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+      <c r="A74" s="19" t="inlineStr">
         <is>
           <t>Legend: pale-yellow cells are yours to type into; white cells hold formulas -- please don't overwrite them.</t>
         </is>

</xml_diff>

<commit_message>
Tie quarterly refill target to P_track instead of a frozen snapshot
The Recommended Transfer formula previously compared each of the 40
quarterly rows against $B$3, a single dollar figure computed once from
today's net worth. That meant the percentage target was effectively frozen
at today's dollar value for the entire 10-year preview instead of tracking
projected portfolio growth.

Added a "Target Safety Anchor Balance (This Year)" column that scales the
Safety Anchor % against that year's P_track (the hurdle model's own
projected wealth trajectory) instead, so the target grows year over year
consistent with the rest of the model. B3 remains as a live "today" snapshot
for reference. Updated the Documentation glossary to match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/household_portfolio_engine.xlsx
+++ b/household_portfolio_engine.xlsx
@@ -935,7 +935,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="38" customHeight="1">
+    <row r="40" ht="68" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
           <t>Safety Anchor</t>
@@ -943,7 +943,7 @@
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>The G Fund cash buffer this engine tries to maintain, expressed as a percentage of total net worth (set on The_Refill_Engine).</t>
+          <t>The G Fund cash buffer this engine tries to maintain, set as a percentage (on The_Refill_Engine). That percentage is applied to each year's projected wealth (P_track), not to today's balance -- so the dollar target grows over time along with the hurdle model instead of staying pinned to today's net worth.</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1671,6 +1671,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1697,7 +1698,7 @@
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>Target Safety Anchor Balance ($)</t>
+          <t>Target Safety Anchor Balance Today ($)</t>
         </is>
       </c>
       <c r="B3" s="22">
@@ -1708,7 +1709,7 @@
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
-          <t>Sequence-of-Returns-Risk (SRR) Shield: the Safety Anchor Target % above controls how large a G Fund cash buffer this engine tries to maintain, so equities are never forced to sell at a loss to fund living expenses. Raise or lower it to fit your risk tolerance.</t>
+          <t>Sequence-of-Returns-Risk (SRR) Shield: the Safety Anchor Target % above controls how large a G Fund cash buffer this engine tries to maintain, so equities are never forced to sell at a loss to fund living expenses. Raise or lower it to fit your risk tolerance. Note: B3 is only a snapshot of today's target -- the Quarterly Refill Engine below scales this same percentage against each year's projected wealth (P_track, from the hurdle model further down this tab) via its own 'Target Safety Anchor Balance (This Year)' column, so the goal grows over time rather than staying pinned to today's balance.</t>
         </is>
       </c>
     </row>
@@ -1726,6 +1727,7 @@
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
@@ -1766,6 +1768,11 @@
       <c r="H7" s="11" t="inlineStr">
         <is>
           <t>G Fund Balance (End of Qtr, Projected)</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Target Safety Anchor Balance (This Year)</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1798,7 @@
         <v/>
       </c>
       <c r="F8" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D8)),MAX(0,$B$3-E8),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D8)),MAX(0,I8-E8),0)</f>
         <v/>
       </c>
       <c r="G8" s="31" t="n"/>
@@ -1799,6 +1806,10 @@
         <f>E8-C8+IF(G8="",F8,G8)</f>
         <v/>
       </c>
+      <c r="I8" s="28">
+        <f>$B$2*D52</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="14" t="n">
@@ -1822,7 +1833,7 @@
         <v/>
       </c>
       <c r="F9" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D9)),MAX(0,$B$3-E9),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D9)),MAX(0,I9-E9),0)</f>
         <v/>
       </c>
       <c r="G9" s="18" t="n"/>
@@ -1830,6 +1841,10 @@
         <f>E9-C9+IF(G9="",F9,G9)</f>
         <v/>
       </c>
+      <c r="I9" s="17">
+        <f>$B$2*D52</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="14" t="n">
@@ -1853,7 +1868,7 @@
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D10)),MAX(0,$B$3-E10),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D10)),MAX(0,I10-E10),0)</f>
         <v/>
       </c>
       <c r="G10" s="18" t="n"/>
@@ -1861,6 +1876,10 @@
         <f>E10-C10+IF(G10="",F10,G10)</f>
         <v/>
       </c>
+      <c r="I10" s="17">
+        <f>$B$2*D52</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="14" t="n">
@@ -1884,7 +1903,7 @@
         <v/>
       </c>
       <c r="F11" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D11)),MAX(0,$B$3-E11),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D11)),MAX(0,I11-E11),0)</f>
         <v/>
       </c>
       <c r="G11" s="18" t="n"/>
@@ -1892,6 +1911,10 @@
         <f>E11-C11+IF(G11="",F11,G11)</f>
         <v/>
       </c>
+      <c r="I11" s="17">
+        <f>$B$2*D52</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="26" t="n">
@@ -1915,7 +1938,7 @@
         <v/>
       </c>
       <c r="F12" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D12)),MAX(0,$B$3-E12),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D12)),MAX(0,I12-E12),0)</f>
         <v/>
       </c>
       <c r="G12" s="31" t="n"/>
@@ -1923,6 +1946,10 @@
         <f>E12-C12+IF(G12="",F12,G12)</f>
         <v/>
       </c>
+      <c r="I12" s="28">
+        <f>$B$2*D53</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="14" t="n">
@@ -1946,7 +1973,7 @@
         <v/>
       </c>
       <c r="F13" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D13)),MAX(0,$B$3-E13),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D13)),MAX(0,I13-E13),0)</f>
         <v/>
       </c>
       <c r="G13" s="18" t="n"/>
@@ -1954,6 +1981,10 @@
         <f>E13-C13+IF(G13="",F13,G13)</f>
         <v/>
       </c>
+      <c r="I13" s="17">
+        <f>$B$2*D53</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="14" t="n">
@@ -1977,7 +2008,7 @@
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D14)),MAX(0,$B$3-E14),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D14)),MAX(0,I14-E14),0)</f>
         <v/>
       </c>
       <c r="G14" s="18" t="n"/>
@@ -1985,6 +2016,10 @@
         <f>E14-C14+IF(G14="",F14,G14)</f>
         <v/>
       </c>
+      <c r="I14" s="17">
+        <f>$B$2*D53</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="14" t="n">
@@ -2008,7 +2043,7 @@
         <v/>
       </c>
       <c r="F15" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D15)),MAX(0,$B$3-E15),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D15)),MAX(0,I15-E15),0)</f>
         <v/>
       </c>
       <c r="G15" s="18" t="n"/>
@@ -2016,6 +2051,10 @@
         <f>E15-C15+IF(G15="",F15,G15)</f>
         <v/>
       </c>
+      <c r="I15" s="17">
+        <f>$B$2*D53</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="26" t="n">
@@ -2039,7 +2078,7 @@
         <v/>
       </c>
       <c r="F16" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D16)),MAX(0,$B$3-E16),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D16)),MAX(0,I16-E16),0)</f>
         <v/>
       </c>
       <c r="G16" s="31" t="n"/>
@@ -2047,6 +2086,10 @@
         <f>E16-C16+IF(G16="",F16,G16)</f>
         <v/>
       </c>
+      <c r="I16" s="28">
+        <f>$B$2*D54</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="14" t="n">
@@ -2070,7 +2113,7 @@
         <v/>
       </c>
       <c r="F17" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D17)),MAX(0,$B$3-E17),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D17)),MAX(0,I17-E17),0)</f>
         <v/>
       </c>
       <c r="G17" s="18" t="n"/>
@@ -2078,6 +2121,10 @@
         <f>E17-C17+IF(G17="",F17,G17)</f>
         <v/>
       </c>
+      <c r="I17" s="17">
+        <f>$B$2*D54</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="14" t="n">
@@ -2101,7 +2148,7 @@
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D18)),MAX(0,$B$3-E18),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D18)),MAX(0,I18-E18),0)</f>
         <v/>
       </c>
       <c r="G18" s="18" t="n"/>
@@ -2109,6 +2156,10 @@
         <f>E18-C18+IF(G18="",F18,G18)</f>
         <v/>
       </c>
+      <c r="I18" s="17">
+        <f>$B$2*D54</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="14" t="n">
@@ -2132,7 +2183,7 @@
         <v/>
       </c>
       <c r="F19" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D19)),MAX(0,$B$3-E19),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D19)),MAX(0,I19-E19),0)</f>
         <v/>
       </c>
       <c r="G19" s="18" t="n"/>
@@ -2140,6 +2191,10 @@
         <f>E19-C19+IF(G19="",F19,G19)</f>
         <v/>
       </c>
+      <c r="I19" s="17">
+        <f>$B$2*D54</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="26" t="n">
@@ -2163,7 +2218,7 @@
         <v/>
       </c>
       <c r="F20" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D20)),MAX(0,$B$3-E20),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D20)),MAX(0,I20-E20),0)</f>
         <v/>
       </c>
       <c r="G20" s="31" t="n"/>
@@ -2171,6 +2226,10 @@
         <f>E20-C20+IF(G20="",F20,G20)</f>
         <v/>
       </c>
+      <c r="I20" s="28">
+        <f>$B$2*D55</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="14" t="n">
@@ -2194,7 +2253,7 @@
         <v/>
       </c>
       <c r="F21" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D21)),MAX(0,$B$3-E21),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D21)),MAX(0,I21-E21),0)</f>
         <v/>
       </c>
       <c r="G21" s="18" t="n"/>
@@ -2202,6 +2261,10 @@
         <f>E21-C21+IF(G21="",F21,G21)</f>
         <v/>
       </c>
+      <c r="I21" s="17">
+        <f>$B$2*D55</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="14" t="n">
@@ -2225,7 +2288,7 @@
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D22)),MAX(0,$B$3-E22),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D22)),MAX(0,I22-E22),0)</f>
         <v/>
       </c>
       <c r="G22" s="18" t="n"/>
@@ -2233,6 +2296,10 @@
         <f>E22-C22+IF(G22="",F22,G22)</f>
         <v/>
       </c>
+      <c r="I22" s="17">
+        <f>$B$2*D55</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="14" t="n">
@@ -2256,7 +2323,7 @@
         <v/>
       </c>
       <c r="F23" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D23)),MAX(0,$B$3-E23),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D23)),MAX(0,I23-E23),0)</f>
         <v/>
       </c>
       <c r="G23" s="18" t="n"/>
@@ -2264,6 +2331,10 @@
         <f>E23-C23+IF(G23="",F23,G23)</f>
         <v/>
       </c>
+      <c r="I23" s="17">
+        <f>$B$2*D55</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="26" t="n">
@@ -2287,7 +2358,7 @@
         <v/>
       </c>
       <c r="F24" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D24)),MAX(0,$B$3-E24),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D24)),MAX(0,I24-E24),0)</f>
         <v/>
       </c>
       <c r="G24" s="31" t="n"/>
@@ -2295,6 +2366,10 @@
         <f>E24-C24+IF(G24="",F24,G24)</f>
         <v/>
       </c>
+      <c r="I24" s="28">
+        <f>$B$2*D56</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="14" t="n">
@@ -2318,7 +2393,7 @@
         <v/>
       </c>
       <c r="F25" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D25)),MAX(0,$B$3-E25),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D25)),MAX(0,I25-E25),0)</f>
         <v/>
       </c>
       <c r="G25" s="18" t="n"/>
@@ -2326,6 +2401,10 @@
         <f>E25-C25+IF(G25="",F25,G25)</f>
         <v/>
       </c>
+      <c r="I25" s="17">
+        <f>$B$2*D56</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="14" t="n">
@@ -2349,7 +2428,7 @@
         <v/>
       </c>
       <c r="F26" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D26)),MAX(0,$B$3-E26),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D26)),MAX(0,I26-E26),0)</f>
         <v/>
       </c>
       <c r="G26" s="18" t="n"/>
@@ -2357,6 +2436,10 @@
         <f>E26-C26+IF(G26="",F26,G26)</f>
         <v/>
       </c>
+      <c r="I26" s="17">
+        <f>$B$2*D56</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="14" t="n">
@@ -2380,7 +2463,7 @@
         <v/>
       </c>
       <c r="F27" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D27)),MAX(0,$B$3-E27),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D27)),MAX(0,I27-E27),0)</f>
         <v/>
       </c>
       <c r="G27" s="18" t="n"/>
@@ -2388,6 +2471,10 @@
         <f>E27-C27+IF(G27="",F27,G27)</f>
         <v/>
       </c>
+      <c r="I27" s="17">
+        <f>$B$2*D56</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="26" t="n">
@@ -2411,7 +2498,7 @@
         <v/>
       </c>
       <c r="F28" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D28)),MAX(0,$B$3-E28),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D28)),MAX(0,I28-E28),0)</f>
         <v/>
       </c>
       <c r="G28" s="31" t="n"/>
@@ -2419,6 +2506,10 @@
         <f>E28-C28+IF(G28="",F28,G28)</f>
         <v/>
       </c>
+      <c r="I28" s="28">
+        <f>$B$2*D57</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="14" t="n">
@@ -2442,7 +2533,7 @@
         <v/>
       </c>
       <c r="F29" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D29)),MAX(0,$B$3-E29),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D29)),MAX(0,I29-E29),0)</f>
         <v/>
       </c>
       <c r="G29" s="18" t="n"/>
@@ -2450,6 +2541,10 @@
         <f>E29-C29+IF(G29="",F29,G29)</f>
         <v/>
       </c>
+      <c r="I29" s="17">
+        <f>$B$2*D57</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="14" t="n">
@@ -2473,7 +2568,7 @@
         <v/>
       </c>
       <c r="F30" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D30)),MAX(0,$B$3-E30),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D30)),MAX(0,I30-E30),0)</f>
         <v/>
       </c>
       <c r="G30" s="18" t="n"/>
@@ -2481,6 +2576,10 @@
         <f>E30-C30+IF(G30="",F30,G30)</f>
         <v/>
       </c>
+      <c r="I30" s="17">
+        <f>$B$2*D57</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="14" t="n">
@@ -2504,7 +2603,7 @@
         <v/>
       </c>
       <c r="F31" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D31)),MAX(0,$B$3-E31),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D31)),MAX(0,I31-E31),0)</f>
         <v/>
       </c>
       <c r="G31" s="18" t="n"/>
@@ -2512,6 +2611,10 @@
         <f>E31-C31+IF(G31="",F31,G31)</f>
         <v/>
       </c>
+      <c r="I31" s="17">
+        <f>$B$2*D57</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="26" t="n">
@@ -2535,7 +2638,7 @@
         <v/>
       </c>
       <c r="F32" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D32)),MAX(0,$B$3-E32),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D32)),MAX(0,I32-E32),0)</f>
         <v/>
       </c>
       <c r="G32" s="31" t="n"/>
@@ -2543,6 +2646,10 @@
         <f>E32-C32+IF(G32="",F32,G32)</f>
         <v/>
       </c>
+      <c r="I32" s="28">
+        <f>$B$2*D58</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="14" t="n">
@@ -2566,7 +2673,7 @@
         <v/>
       </c>
       <c r="F33" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D33)),MAX(0,$B$3-E33),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D33)),MAX(0,I33-E33),0)</f>
         <v/>
       </c>
       <c r="G33" s="18" t="n"/>
@@ -2574,6 +2681,10 @@
         <f>E33-C33+IF(G33="",F33,G33)</f>
         <v/>
       </c>
+      <c r="I33" s="17">
+        <f>$B$2*D58</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="14" t="n">
@@ -2597,7 +2708,7 @@
         <v/>
       </c>
       <c r="F34" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D34)),MAX(0,$B$3-E34),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D34)),MAX(0,I34-E34),0)</f>
         <v/>
       </c>
       <c r="G34" s="18" t="n"/>
@@ -2605,6 +2716,10 @@
         <f>E34-C34+IF(G34="",F34,G34)</f>
         <v/>
       </c>
+      <c r="I34" s="17">
+        <f>$B$2*D58</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="14" t="n">
@@ -2628,7 +2743,7 @@
         <v/>
       </c>
       <c r="F35" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D35)),MAX(0,$B$3-E35),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D35)),MAX(0,I35-E35),0)</f>
         <v/>
       </c>
       <c r="G35" s="18" t="n"/>
@@ -2636,6 +2751,10 @@
         <f>E35-C35+IF(G35="",F35,G35)</f>
         <v/>
       </c>
+      <c r="I35" s="17">
+        <f>$B$2*D58</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="26" t="n">
@@ -2659,7 +2778,7 @@
         <v/>
       </c>
       <c r="F36" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D36)),MAX(0,$B$3-E36),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D36)),MAX(0,I36-E36),0)</f>
         <v/>
       </c>
       <c r="G36" s="31" t="n"/>
@@ -2667,6 +2786,10 @@
         <f>E36-C36+IF(G36="",F36,G36)</f>
         <v/>
       </c>
+      <c r="I36" s="28">
+        <f>$B$2*D59</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="14" t="n">
@@ -2690,7 +2813,7 @@
         <v/>
       </c>
       <c r="F37" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D37)),MAX(0,$B$3-E37),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D37)),MAX(0,I37-E37),0)</f>
         <v/>
       </c>
       <c r="G37" s="18" t="n"/>
@@ -2698,6 +2821,10 @@
         <f>E37-C37+IF(G37="",F37,G37)</f>
         <v/>
       </c>
+      <c r="I37" s="17">
+        <f>$B$2*D59</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="14" t="n">
@@ -2721,7 +2848,7 @@
         <v/>
       </c>
       <c r="F38" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D38)),MAX(0,$B$3-E38),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D38)),MAX(0,I38-E38),0)</f>
         <v/>
       </c>
       <c r="G38" s="18" t="n"/>
@@ -2729,6 +2856,10 @@
         <f>E38-C38+IF(G38="",F38,G38)</f>
         <v/>
       </c>
+      <c r="I38" s="17">
+        <f>$B$2*D59</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="14" t="n">
@@ -2752,7 +2883,7 @@
         <v/>
       </c>
       <c r="F39" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D39)),MAX(0,$B$3-E39),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D39)),MAX(0,I39-E39),0)</f>
         <v/>
       </c>
       <c r="G39" s="18" t="n"/>
@@ -2760,6 +2891,10 @@
         <f>E39-C39+IF(G39="",F39,G39)</f>
         <v/>
       </c>
+      <c r="I39" s="17">
+        <f>$B$2*D59</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="26" t="n">
@@ -2783,7 +2918,7 @@
         <v/>
       </c>
       <c r="F40" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D40)),MAX(0,$B$3-E40),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D40)),MAX(0,I40-E40),0)</f>
         <v/>
       </c>
       <c r="G40" s="31" t="n"/>
@@ -2791,6 +2926,10 @@
         <f>E40-C40+IF(G40="",F40,G40)</f>
         <v/>
       </c>
+      <c r="I40" s="28">
+        <f>$B$2*D60</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="14" t="n">
@@ -2814,7 +2953,7 @@
         <v/>
       </c>
       <c r="F41" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D41)),MAX(0,$B$3-E41),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D41)),MAX(0,I41-E41),0)</f>
         <v/>
       </c>
       <c r="G41" s="18" t="n"/>
@@ -2822,6 +2961,10 @@
         <f>E41-C41+IF(G41="",F41,G41)</f>
         <v/>
       </c>
+      <c r="I41" s="17">
+        <f>$B$2*D60</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="14" t="n">
@@ -2845,7 +2988,7 @@
         <v/>
       </c>
       <c r="F42" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D42)),MAX(0,$B$3-E42),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D42)),MAX(0,I42-E42),0)</f>
         <v/>
       </c>
       <c r="G42" s="18" t="n"/>
@@ -2853,6 +2996,10 @@
         <f>E42-C42+IF(G42="",F42,G42)</f>
         <v/>
       </c>
+      <c r="I42" s="17">
+        <f>$B$2*D60</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="14" t="n">
@@ -2876,7 +3023,7 @@
         <v/>
       </c>
       <c r="F43" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D43)),MAX(0,$B$3-E43),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D43)),MAX(0,I43-E43),0)</f>
         <v/>
       </c>
       <c r="G43" s="18" t="n"/>
@@ -2884,6 +3031,10 @@
         <f>E43-C43+IF(G43="",F43,G43)</f>
         <v/>
       </c>
+      <c r="I43" s="17">
+        <f>$B$2*D60</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="26" t="n">
@@ -2907,7 +3058,7 @@
         <v/>
       </c>
       <c r="F44" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D44)),MAX(0,$B$3-E44),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D44)),MAX(0,I44-E44),0)</f>
         <v/>
       </c>
       <c r="G44" s="31" t="n"/>
@@ -2915,6 +3066,10 @@
         <f>E44-C44+IF(G44="",F44,G44)</f>
         <v/>
       </c>
+      <c r="I44" s="28">
+        <f>$B$2*D61</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="14" t="n">
@@ -2938,7 +3093,7 @@
         <v/>
       </c>
       <c r="F45" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D45)),MAX(0,$B$3-E45),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D45)),MAX(0,I45-E45),0)</f>
         <v/>
       </c>
       <c r="G45" s="18" t="n"/>
@@ -2946,6 +3101,10 @@
         <f>E45-C45+IF(G45="",F45,G45)</f>
         <v/>
       </c>
+      <c r="I45" s="17">
+        <f>$B$2*D61</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="14" t="n">
@@ -2969,7 +3128,7 @@
         <v/>
       </c>
       <c r="F46" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D46)),MAX(0,$B$3-E46),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D46)),MAX(0,I46-E46),0)</f>
         <v/>
       </c>
       <c r="G46" s="18" t="n"/>
@@ -2977,6 +3136,10 @@
         <f>E46-C46+IF(G46="",F46,G46)</f>
         <v/>
       </c>
+      <c r="I46" s="17">
+        <f>$B$2*D61</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="28" customHeight="1">
       <c r="A47" s="14" t="n">
@@ -3000,12 +3163,16 @@
         <v/>
       </c>
       <c r="F47" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D47)),MAX(0,$B$3-E47),0)</f>
+        <f>IF(ISNUMBER(SEARCH("GOOD",D47)),MAX(0,I47-E47),0)</f>
         <v/>
       </c>
       <c r="G47" s="18" t="n"/>
       <c r="H47" s="17">
         <f>E47-C47+IF(G47="",F47,G47)</f>
+        <v/>
+      </c>
+      <c r="I47" s="17">
+        <f>$B$2*D61</f>
         <v/>
       </c>
     </row>
@@ -3359,7 +3526,7 @@
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="B70:E72"/>
     <mergeCell ref="A63:C63"/>
-    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A6:I6"/>
   </mergeCells>
   <conditionalFormatting sqref="B70:B72">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>

<commit_message>
Switch Safety Anchor % from a flat input to a step function
Replaces the single "Safety Anchor Target %" input with a step function
matching the SRR literature more literally: an elevated Red Zone % through
the first N years of retirement, then a lower Post-Red-Zone %, rather than
a flat percentage or a smooth age-based taper. Deliberately clock-driven
(keyed off Retirement Start Year / Age at Retirement Start / Red Zone
Length) rather than expense-driven, so it isn't perturbed by month-to-month
spending variability during the early years.

New inputs on The_Refill_Engine: Retirement Start Year, Age at Retirement
Start, Red Zone Length (Years), Red Zone Target %, Post-Red-Zone Target %.
The Annual SRR Hurdle Model gets a new "Safety Anchor % (This Year)" column
implementing the step, which now drives the Quarterly Refill Engine's
per-year target instead of a flat percentage. Row 8 keeps a live "today"
snapshot for quick reference.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/household_portfolio_engine.xlsx
+++ b/household_portfolio_engine.xlsx
@@ -147,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -183,6 +183,7 @@
     <xf numFmtId="164" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -608,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -935,7 +936,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="68" customHeight="1">
+    <row r="40" ht="98" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
           <t>Safety Anchor</t>
@@ -943,41 +944,53 @@
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>The G Fund cash buffer this engine tries to maintain, set as a percentage (on The_Refill_Engine). That percentage is applied to each year's projected wealth (P_track), not to today's balance -- so the dollar target grows over time along with the hurdle model instead of staying pinned to today's net worth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="38" customHeight="1">
+          <t>The G Fund cash buffer this engine tries to maintain. Set as a step function (on The_Refill_Engine): a higher percentage through the SRR "red zone" -- the first several years of retirement -- then a lower one afterward. That percentage is applied each year to that year's projected wealth (P_track), not to today's balance, so the dollar target still grows within each step instead of staying pinned to today's net worth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="53" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>Conduit</t>
+          <t>Red Zone</t>
         </is>
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>A Traditional IRA used as a pass-through for pre-tax rollovers back into the TSP.</t>
+          <t>The first several years of retirement, when a bad sequence of market returns does the most lasting damage to a portfolio (SRR risk is heavily front-loaded). The Safety Anchor holds a higher percentage during this window.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="38" customHeight="1">
       <c r="A42" s="12" t="inlineStr">
         <is>
+          <t>Conduit</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>A Traditional IRA used as a pass-through for pre-tax rollovers back into the TSP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="38" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
           <t>Rollover</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B43" s="13" t="inlineStr">
         <is>
           <t>A pre-tax transfer of funds between retirement accounts (e.g. Traditional IRA to TSP) that doesn't trigger a taxable distribution.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="23" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="44" ht="23" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>Allocation Mix</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>Each account's share of total household net worth, shown on Account_Tracker.</t>
         </is>
@@ -1660,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1688,319 +1701,195 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t>Safety Anchor Target % (of Net Worth)</t>
+          <t>Retirement Start Year</t>
         </is>
       </c>
       <c r="B2" s="25" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Age at Retirement Start</t>
+        </is>
+      </c>
+      <c r="B3" s="25" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Red Zone Length (Years)</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Red Zone Target % (elevated, early retirement)</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="n">
         <v>0.35</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Post-Red-Zone Target % (steady state)</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Current Safety Anchor %</t>
+        </is>
+      </c>
+      <c r="B7" s="23">
+        <f>IF(YEAR(TODAY())-B2&lt;B4,B5,B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Target Safety Anchor Balance Today ($)</t>
         </is>
       </c>
-      <c r="B3" s="22">
-        <f>B1*B2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>Sequence-of-Returns-Risk (SRR) Shield: the Safety Anchor Target % above controls how large a G Fund cash buffer this engine tries to maintain, so equities are never forced to sell at a loss to fund living expenses. Raise or lower it to fit your risk tolerance. Note: B3 is only a snapshot of today's target -- the Quarterly Refill Engine below scales this same percentage against each year's projected wealth (P_track, from the hurdle model further down this tab) via its own 'Target Safety Anchor Balance (This Year)' column, so the goal grows over time rather than staying pinned to today's balance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="B8" s="22">
+        <f>B1*B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Sequence-of-Returns-Risk (SRR) Shield: this engine uses a step function, not a flat percentage. SRR is concentrated in the first years of retirement (the "red zone"), when a bad sequence does the most damage; research supports holding a larger safety anchor through that window, then a smaller one afterward, rather than raising it further with age. Each year's actual target -- Red Zone % while Age &lt; Age-at-Retirement + Red-Zone-Length, Post-Red-Zone % after -- is computed per-year in the Annual SRR Hurdle Model below and drives the Quarterly Refill Engine's 'Target Safety Anchor Balance (This Year)' column. Row 8 above is only a live snapshot of today's applicable target for quick reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>THE QUARTERLY REFILL ENGINE — PRIMARY OUTPUT: RECOMMENDED TSP TOP-UP TRANSFER</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>Quarterly Outflow (W_q)</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Annual Performance Signal</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>G Fund Balance (Start of Qtr)</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>Recommended Transfer This Quarter</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>Actual Transferred (Log It Here)</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>G Fund Balance (End of Qtr, Projected)</t>
         </is>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>Target Safety Anchor Balance (This Year)</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="26" t="n">
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="27" t="n">
         <v>2026</v>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C8" s="28">
+      <c r="C13" s="29">
         <f>SUM('Variables_And_Log'!F3:H3)</f>
         <v/>
       </c>
-      <c r="D8" s="29">
-        <f>E52</f>
-        <v/>
-      </c>
-      <c r="E8" s="28">
+      <c r="D13" s="30">
+        <f>E57</f>
+        <v/>
+      </c>
+      <c r="E13" s="29">
         <f>'Account_Tracker'!$C$2</f>
         <v/>
       </c>
-      <c r="F8" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D8)),MAX(0,I8-E8),0)</f>
-        <v/>
-      </c>
-      <c r="G8" s="31" t="n"/>
-      <c r="H8" s="28">
-        <f>E8-C8+IF(G8="",F8,G8)</f>
-        <v/>
-      </c>
-      <c r="I8" s="28">
-        <f>$B$2*D52</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="14" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C9" s="17">
-        <f>SUM('Variables_And_Log'!I3:K3)</f>
-        <v/>
-      </c>
-      <c r="D9" s="32">
-        <f>E52</f>
-        <v/>
-      </c>
-      <c r="E9" s="17">
-        <f>H8</f>
-        <v/>
-      </c>
-      <c r="F9" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D9)),MAX(0,I9-E9),0)</f>
-        <v/>
-      </c>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="17">
-        <f>E9-C9+IF(G9="",F9,G9)</f>
-        <v/>
-      </c>
-      <c r="I9" s="17">
-        <f>$B$2*D52</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="14" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="C10" s="17">
-        <f>SUM('Variables_And_Log'!L3:N3)</f>
-        <v/>
-      </c>
-      <c r="D10" s="32">
-        <f>E52</f>
-        <v/>
-      </c>
-      <c r="E10" s="17">
-        <f>H9</f>
-        <v/>
-      </c>
-      <c r="F10" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D10)),MAX(0,I10-E10),0)</f>
-        <v/>
-      </c>
-      <c r="G10" s="18" t="n"/>
-      <c r="H10" s="17">
-        <f>E10-C10+IF(G10="",F10,G10)</f>
-        <v/>
-      </c>
-      <c r="I10" s="17">
-        <f>$B$2*D52</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="14" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="C11" s="17">
-        <f>SUM('Variables_And_Log'!O3:Q3)</f>
-        <v/>
-      </c>
-      <c r="D11" s="32">
-        <f>E52</f>
-        <v/>
-      </c>
-      <c r="E11" s="17">
-        <f>H10</f>
-        <v/>
-      </c>
-      <c r="F11" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D11)),MAX(0,I11-E11),0)</f>
-        <v/>
-      </c>
-      <c r="G11" s="18" t="n"/>
-      <c r="H11" s="17">
-        <f>E11-C11+IF(G11="",F11,G11)</f>
-        <v/>
-      </c>
-      <c r="I11" s="17">
-        <f>$B$2*D52</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="26" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="C12" s="28">
-        <f>SUM('Variables_And_Log'!F4:H4)</f>
-        <v/>
-      </c>
-      <c r="D12" s="29">
-        <f>E53</f>
-        <v/>
-      </c>
-      <c r="E12" s="28">
-        <f>H11</f>
-        <v/>
-      </c>
-      <c r="F12" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D12)),MAX(0,I12-E12),0)</f>
-        <v/>
-      </c>
-      <c r="G12" s="31" t="n"/>
-      <c r="H12" s="28">
-        <f>E12-C12+IF(G12="",F12,G12)</f>
-        <v/>
-      </c>
-      <c r="I12" s="28">
-        <f>$B$2*D53</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="14" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C13" s="17">
-        <f>SUM('Variables_And_Log'!I4:K4)</f>
-        <v/>
-      </c>
-      <c r="D13" s="32">
-        <f>E53</f>
-        <v/>
-      </c>
-      <c r="E13" s="17">
-        <f>H12</f>
-        <v/>
-      </c>
-      <c r="F13" s="22">
+      <c r="F13" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D13)),MAX(0,I13-E13),0)</f>
         <v/>
       </c>
-      <c r="G13" s="18" t="n"/>
-      <c r="H13" s="17">
+      <c r="G13" s="32" t="n"/>
+      <c r="H13" s="29">
         <f>E13-C13+IF(G13="",F13,G13)</f>
         <v/>
       </c>
-      <c r="I13" s="17">
-        <f>$B$2*D53</f>
+      <c r="I13" s="29">
+        <f>F57*D57</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="14" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C14" s="17">
-        <f>SUM('Variables_And_Log'!L4:N4)</f>
-        <v/>
-      </c>
-      <c r="D14" s="32">
-        <f>E53</f>
+        <f>SUM('Variables_And_Log'!I3:K3)</f>
+        <v/>
+      </c>
+      <c r="D14" s="33">
+        <f>E57</f>
         <v/>
       </c>
       <c r="E14" s="17">
@@ -2017,25 +1906,25 @@
         <v/>
       </c>
       <c r="I14" s="17">
-        <f>$B$2*D53</f>
+        <f>F57*D57</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="14" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C15" s="17">
-        <f>SUM('Variables_And_Log'!O4:Q4)</f>
-        <v/>
-      </c>
-      <c r="D15" s="32">
-        <f>E53</f>
+        <f>SUM('Variables_And_Log'!L3:N3)</f>
+        <v/>
+      </c>
+      <c r="D15" s="33">
+        <f>E57</f>
         <v/>
       </c>
       <c r="E15" s="17">
@@ -2052,95 +1941,95 @@
         <v/>
       </c>
       <c r="I15" s="17">
-        <f>$B$2*D53</f>
+        <f>F57*D57</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="26" t="n">
-        <v>2028</v>
-      </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="A16" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C16" s="17">
+        <f>SUM('Variables_And_Log'!O3:Q3)</f>
+        <v/>
+      </c>
+      <c r="D16" s="33">
+        <f>E57</f>
+        <v/>
+      </c>
+      <c r="E16" s="17">
+        <f>H15</f>
+        <v/>
+      </c>
+      <c r="F16" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D16)),MAX(0,I16-E16),0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="17">
+        <f>E16-C16+IF(G16="",F16,G16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="17">
+        <f>F57*D57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="27" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C16" s="28">
-        <f>SUM('Variables_And_Log'!F5:H5)</f>
-        <v/>
-      </c>
-      <c r="D16" s="29">
-        <f>E54</f>
-        <v/>
-      </c>
-      <c r="E16" s="28">
-        <f>H15</f>
-        <v/>
-      </c>
-      <c r="F16" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D16)),MAX(0,I16-E16),0)</f>
-        <v/>
-      </c>
-      <c r="G16" s="31" t="n"/>
-      <c r="H16" s="28">
-        <f>E16-C16+IF(G16="",F16,G16)</f>
-        <v/>
-      </c>
-      <c r="I16" s="28">
-        <f>$B$2*D54</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="14" t="n">
-        <v>2028</v>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C17" s="17">
-        <f>SUM('Variables_And_Log'!I5:K5)</f>
-        <v/>
-      </c>
-      <c r="D17" s="32">
-        <f>E54</f>
-        <v/>
-      </c>
-      <c r="E17" s="17">
+      <c r="C17" s="29">
+        <f>SUM('Variables_And_Log'!F4:H4)</f>
+        <v/>
+      </c>
+      <c r="D17" s="30">
+        <f>E58</f>
+        <v/>
+      </c>
+      <c r="E17" s="29">
         <f>H16</f>
         <v/>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D17)),MAX(0,I17-E17),0)</f>
         <v/>
       </c>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="17">
+      <c r="G17" s="32" t="n"/>
+      <c r="H17" s="29">
         <f>E17-C17+IF(G17="",F17,G17)</f>
         <v/>
       </c>
-      <c r="I17" s="17">
-        <f>$B$2*D54</f>
+      <c r="I17" s="29">
+        <f>F58*D58</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="14" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C18" s="17">
-        <f>SUM('Variables_And_Log'!L5:N5)</f>
-        <v/>
-      </c>
-      <c r="D18" s="32">
-        <f>E54</f>
+        <f>SUM('Variables_And_Log'!I4:K4)</f>
+        <v/>
+      </c>
+      <c r="D18" s="33">
+        <f>E58</f>
         <v/>
       </c>
       <c r="E18" s="17">
@@ -2157,25 +2046,25 @@
         <v/>
       </c>
       <c r="I18" s="17">
-        <f>$B$2*D54</f>
+        <f>F58*D58</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="14" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C19" s="17">
-        <f>SUM('Variables_And_Log'!O5:Q5)</f>
-        <v/>
-      </c>
-      <c r="D19" s="32">
-        <f>E54</f>
+        <f>SUM('Variables_And_Log'!L4:N4)</f>
+        <v/>
+      </c>
+      <c r="D19" s="33">
+        <f>E58</f>
         <v/>
       </c>
       <c r="E19" s="17">
@@ -2192,95 +2081,95 @@
         <v/>
       </c>
       <c r="I19" s="17">
-        <f>$B$2*D54</f>
+        <f>F58*D58</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="26" t="n">
-        <v>2029</v>
-      </c>
-      <c r="B20" s="27" t="inlineStr">
+      <c r="A20" s="14" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C20" s="17">
+        <f>SUM('Variables_And_Log'!O4:Q4)</f>
+        <v/>
+      </c>
+      <c r="D20" s="33">
+        <f>E58</f>
+        <v/>
+      </c>
+      <c r="E20" s="17">
+        <f>H19</f>
+        <v/>
+      </c>
+      <c r="F20" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D20)),MAX(0,I20-E20),0)</f>
+        <v/>
+      </c>
+      <c r="G20" s="18" t="n"/>
+      <c r="H20" s="17">
+        <f>E20-C20+IF(G20="",F20,G20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="17">
+        <f>F58*D58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="27" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C20" s="28">
-        <f>SUM('Variables_And_Log'!F6:H6)</f>
-        <v/>
-      </c>
-      <c r="D20" s="29">
-        <f>E55</f>
-        <v/>
-      </c>
-      <c r="E20" s="28">
-        <f>H19</f>
-        <v/>
-      </c>
-      <c r="F20" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D20)),MAX(0,I20-E20),0)</f>
-        <v/>
-      </c>
-      <c r="G20" s="31" t="n"/>
-      <c r="H20" s="28">
-        <f>E20-C20+IF(G20="",F20,G20)</f>
-        <v/>
-      </c>
-      <c r="I20" s="28">
-        <f>$B$2*D55</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="14" t="n">
-        <v>2029</v>
-      </c>
-      <c r="B21" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C21" s="17">
-        <f>SUM('Variables_And_Log'!I6:K6)</f>
-        <v/>
-      </c>
-      <c r="D21" s="32">
-        <f>E55</f>
-        <v/>
-      </c>
-      <c r="E21" s="17">
+      <c r="C21" s="29">
+        <f>SUM('Variables_And_Log'!F5:H5)</f>
+        <v/>
+      </c>
+      <c r="D21" s="30">
+        <f>E59</f>
+        <v/>
+      </c>
+      <c r="E21" s="29">
         <f>H20</f>
         <v/>
       </c>
-      <c r="F21" s="22">
+      <c r="F21" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D21)),MAX(0,I21-E21),0)</f>
         <v/>
       </c>
-      <c r="G21" s="18" t="n"/>
-      <c r="H21" s="17">
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="29">
         <f>E21-C21+IF(G21="",F21,G21)</f>
         <v/>
       </c>
-      <c r="I21" s="17">
-        <f>$B$2*D55</f>
+      <c r="I21" s="29">
+        <f>F59*D59</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="14" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C22" s="17">
-        <f>SUM('Variables_And_Log'!L6:N6)</f>
-        <v/>
-      </c>
-      <c r="D22" s="32">
-        <f>E55</f>
+        <f>SUM('Variables_And_Log'!I5:K5)</f>
+        <v/>
+      </c>
+      <c r="D22" s="33">
+        <f>E59</f>
         <v/>
       </c>
       <c r="E22" s="17">
@@ -2297,25 +2186,25 @@
         <v/>
       </c>
       <c r="I22" s="17">
-        <f>$B$2*D55</f>
+        <f>F59*D59</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="14" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C23" s="17">
-        <f>SUM('Variables_And_Log'!O6:Q6)</f>
-        <v/>
-      </c>
-      <c r="D23" s="32">
-        <f>E55</f>
+        <f>SUM('Variables_And_Log'!L5:N5)</f>
+        <v/>
+      </c>
+      <c r="D23" s="33">
+        <f>E59</f>
         <v/>
       </c>
       <c r="E23" s="17">
@@ -2332,95 +2221,95 @@
         <v/>
       </c>
       <c r="I23" s="17">
-        <f>$B$2*D55</f>
+        <f>F59*D59</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="26" t="n">
-        <v>2030</v>
-      </c>
-      <c r="B24" s="27" t="inlineStr">
+      <c r="A24" s="14" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C24" s="17">
+        <f>SUM('Variables_And_Log'!O5:Q5)</f>
+        <v/>
+      </c>
+      <c r="D24" s="33">
+        <f>E59</f>
+        <v/>
+      </c>
+      <c r="E24" s="17">
+        <f>H23</f>
+        <v/>
+      </c>
+      <c r="F24" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D24)),MAX(0,I24-E24),0)</f>
+        <v/>
+      </c>
+      <c r="G24" s="18" t="n"/>
+      <c r="H24" s="17">
+        <f>E24-C24+IF(G24="",F24,G24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="17">
+        <f>F59*D59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="27" t="n">
+        <v>2029</v>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C24" s="28">
-        <f>SUM('Variables_And_Log'!F7:H7)</f>
-        <v/>
-      </c>
-      <c r="D24" s="29">
-        <f>E56</f>
-        <v/>
-      </c>
-      <c r="E24" s="28">
-        <f>H23</f>
-        <v/>
-      </c>
-      <c r="F24" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D24)),MAX(0,I24-E24),0)</f>
-        <v/>
-      </c>
-      <c r="G24" s="31" t="n"/>
-      <c r="H24" s="28">
-        <f>E24-C24+IF(G24="",F24,G24)</f>
-        <v/>
-      </c>
-      <c r="I24" s="28">
-        <f>$B$2*D56</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="14" t="n">
-        <v>2030</v>
-      </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C25" s="17">
-        <f>SUM('Variables_And_Log'!I7:K7)</f>
-        <v/>
-      </c>
-      <c r="D25" s="32">
-        <f>E56</f>
-        <v/>
-      </c>
-      <c r="E25" s="17">
+      <c r="C25" s="29">
+        <f>SUM('Variables_And_Log'!F6:H6)</f>
+        <v/>
+      </c>
+      <c r="D25" s="30">
+        <f>E60</f>
+        <v/>
+      </c>
+      <c r="E25" s="29">
         <f>H24</f>
         <v/>
       </c>
-      <c r="F25" s="22">
+      <c r="F25" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D25)),MAX(0,I25-E25),0)</f>
         <v/>
       </c>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="17">
+      <c r="G25" s="32" t="n"/>
+      <c r="H25" s="29">
         <f>E25-C25+IF(G25="",F25,G25)</f>
         <v/>
       </c>
-      <c r="I25" s="17">
-        <f>$B$2*D56</f>
+      <c r="I25" s="29">
+        <f>F60*D60</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="14" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C26" s="17">
-        <f>SUM('Variables_And_Log'!L7:N7)</f>
-        <v/>
-      </c>
-      <c r="D26" s="32">
-        <f>E56</f>
+        <f>SUM('Variables_And_Log'!I6:K6)</f>
+        <v/>
+      </c>
+      <c r="D26" s="33">
+        <f>E60</f>
         <v/>
       </c>
       <c r="E26" s="17">
@@ -2437,25 +2326,25 @@
         <v/>
       </c>
       <c r="I26" s="17">
-        <f>$B$2*D56</f>
+        <f>F60*D60</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="14" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C27" s="17">
-        <f>SUM('Variables_And_Log'!O7:Q7)</f>
-        <v/>
-      </c>
-      <c r="D27" s="32">
-        <f>E56</f>
+        <f>SUM('Variables_And_Log'!L6:N6)</f>
+        <v/>
+      </c>
+      <c r="D27" s="33">
+        <f>E60</f>
         <v/>
       </c>
       <c r="E27" s="17">
@@ -2472,95 +2361,95 @@
         <v/>
       </c>
       <c r="I27" s="17">
-        <f>$B$2*D56</f>
+        <f>F60*D60</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="26" t="n">
-        <v>2031</v>
-      </c>
-      <c r="B28" s="27" t="inlineStr">
+      <c r="A28" s="14" t="n">
+        <v>2029</v>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C28" s="17">
+        <f>SUM('Variables_And_Log'!O6:Q6)</f>
+        <v/>
+      </c>
+      <c r="D28" s="33">
+        <f>E60</f>
+        <v/>
+      </c>
+      <c r="E28" s="17">
+        <f>H27</f>
+        <v/>
+      </c>
+      <c r="F28" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D28)),MAX(0,I28-E28),0)</f>
+        <v/>
+      </c>
+      <c r="G28" s="18" t="n"/>
+      <c r="H28" s="17">
+        <f>E28-C28+IF(G28="",F28,G28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="17">
+        <f>F60*D60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="27" t="n">
+        <v>2030</v>
+      </c>
+      <c r="B29" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C28" s="28">
-        <f>SUM('Variables_And_Log'!F8:H8)</f>
-        <v/>
-      </c>
-      <c r="D28" s="29">
-        <f>E57</f>
-        <v/>
-      </c>
-      <c r="E28" s="28">
-        <f>H27</f>
-        <v/>
-      </c>
-      <c r="F28" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D28)),MAX(0,I28-E28),0)</f>
-        <v/>
-      </c>
-      <c r="G28" s="31" t="n"/>
-      <c r="H28" s="28">
-        <f>E28-C28+IF(G28="",F28,G28)</f>
-        <v/>
-      </c>
-      <c r="I28" s="28">
-        <f>$B$2*D57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="14" t="n">
-        <v>2031</v>
-      </c>
-      <c r="B29" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C29" s="17">
-        <f>SUM('Variables_And_Log'!I8:K8)</f>
-        <v/>
-      </c>
-      <c r="D29" s="32">
-        <f>E57</f>
-        <v/>
-      </c>
-      <c r="E29" s="17">
+      <c r="C29" s="29">
+        <f>SUM('Variables_And_Log'!F7:H7)</f>
+        <v/>
+      </c>
+      <c r="D29" s="30">
+        <f>E61</f>
+        <v/>
+      </c>
+      <c r="E29" s="29">
         <f>H28</f>
         <v/>
       </c>
-      <c r="F29" s="22">
+      <c r="F29" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D29)),MAX(0,I29-E29),0)</f>
         <v/>
       </c>
-      <c r="G29" s="18" t="n"/>
-      <c r="H29" s="17">
+      <c r="G29" s="32" t="n"/>
+      <c r="H29" s="29">
         <f>E29-C29+IF(G29="",F29,G29)</f>
         <v/>
       </c>
-      <c r="I29" s="17">
-        <f>$B$2*D57</f>
+      <c r="I29" s="29">
+        <f>F61*D61</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="14" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C30" s="17">
-        <f>SUM('Variables_And_Log'!L8:N8)</f>
-        <v/>
-      </c>
-      <c r="D30" s="32">
-        <f>E57</f>
+        <f>SUM('Variables_And_Log'!I7:K7)</f>
+        <v/>
+      </c>
+      <c r="D30" s="33">
+        <f>E61</f>
         <v/>
       </c>
       <c r="E30" s="17">
@@ -2577,25 +2466,25 @@
         <v/>
       </c>
       <c r="I30" s="17">
-        <f>$B$2*D57</f>
+        <f>F61*D61</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="14" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B31" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C31" s="17">
-        <f>SUM('Variables_And_Log'!O8:Q8)</f>
-        <v/>
-      </c>
-      <c r="D31" s="32">
-        <f>E57</f>
+        <f>SUM('Variables_And_Log'!L7:N7)</f>
+        <v/>
+      </c>
+      <c r="D31" s="33">
+        <f>E61</f>
         <v/>
       </c>
       <c r="E31" s="17">
@@ -2612,95 +2501,95 @@
         <v/>
       </c>
       <c r="I31" s="17">
-        <f>$B$2*D57</f>
+        <f>F61*D61</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="26" t="n">
-        <v>2032</v>
-      </c>
-      <c r="B32" s="27" t="inlineStr">
+      <c r="A32" s="14" t="n">
+        <v>2030</v>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C32" s="17">
+        <f>SUM('Variables_And_Log'!O7:Q7)</f>
+        <v/>
+      </c>
+      <c r="D32" s="33">
+        <f>E61</f>
+        <v/>
+      </c>
+      <c r="E32" s="17">
+        <f>H31</f>
+        <v/>
+      </c>
+      <c r="F32" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D32)),MAX(0,I32-E32),0)</f>
+        <v/>
+      </c>
+      <c r="G32" s="18" t="n"/>
+      <c r="H32" s="17">
+        <f>E32-C32+IF(G32="",F32,G32)</f>
+        <v/>
+      </c>
+      <c r="I32" s="17">
+        <f>F61*D61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="27" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B33" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C32" s="28">
-        <f>SUM('Variables_And_Log'!F9:H9)</f>
-        <v/>
-      </c>
-      <c r="D32" s="29">
-        <f>E58</f>
-        <v/>
-      </c>
-      <c r="E32" s="28">
-        <f>H31</f>
-        <v/>
-      </c>
-      <c r="F32" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D32)),MAX(0,I32-E32),0)</f>
-        <v/>
-      </c>
-      <c r="G32" s="31" t="n"/>
-      <c r="H32" s="28">
-        <f>E32-C32+IF(G32="",F32,G32)</f>
-        <v/>
-      </c>
-      <c r="I32" s="28">
-        <f>$B$2*D58</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="14" t="n">
-        <v>2032</v>
-      </c>
-      <c r="B33" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C33" s="17">
-        <f>SUM('Variables_And_Log'!I9:K9)</f>
-        <v/>
-      </c>
-      <c r="D33" s="32">
-        <f>E58</f>
-        <v/>
-      </c>
-      <c r="E33" s="17">
+      <c r="C33" s="29">
+        <f>SUM('Variables_And_Log'!F8:H8)</f>
+        <v/>
+      </c>
+      <c r="D33" s="30">
+        <f>E62</f>
+        <v/>
+      </c>
+      <c r="E33" s="29">
         <f>H32</f>
         <v/>
       </c>
-      <c r="F33" s="22">
+      <c r="F33" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D33)),MAX(0,I33-E33),0)</f>
         <v/>
       </c>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="17">
+      <c r="G33" s="32" t="n"/>
+      <c r="H33" s="29">
         <f>E33-C33+IF(G33="",F33,G33)</f>
         <v/>
       </c>
-      <c r="I33" s="17">
-        <f>$B$2*D58</f>
+      <c r="I33" s="29">
+        <f>F62*D62</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="14" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B34" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C34" s="17">
-        <f>SUM('Variables_And_Log'!L9:N9)</f>
-        <v/>
-      </c>
-      <c r="D34" s="32">
-        <f>E58</f>
+        <f>SUM('Variables_And_Log'!I8:K8)</f>
+        <v/>
+      </c>
+      <c r="D34" s="33">
+        <f>E62</f>
         <v/>
       </c>
       <c r="E34" s="17">
@@ -2717,25 +2606,25 @@
         <v/>
       </c>
       <c r="I34" s="17">
-        <f>$B$2*D58</f>
+        <f>F62*D62</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="14" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B35" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C35" s="17">
-        <f>SUM('Variables_And_Log'!O9:Q9)</f>
-        <v/>
-      </c>
-      <c r="D35" s="32">
-        <f>E58</f>
+        <f>SUM('Variables_And_Log'!L8:N8)</f>
+        <v/>
+      </c>
+      <c r="D35" s="33">
+        <f>E62</f>
         <v/>
       </c>
       <c r="E35" s="17">
@@ -2752,95 +2641,95 @@
         <v/>
       </c>
       <c r="I35" s="17">
-        <f>$B$2*D58</f>
+        <f>F62*D62</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="26" t="n">
-        <v>2033</v>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
+      <c r="A36" s="14" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B36" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C36" s="17">
+        <f>SUM('Variables_And_Log'!O8:Q8)</f>
+        <v/>
+      </c>
+      <c r="D36" s="33">
+        <f>E62</f>
+        <v/>
+      </c>
+      <c r="E36" s="17">
+        <f>H35</f>
+        <v/>
+      </c>
+      <c r="F36" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D36)),MAX(0,I36-E36),0)</f>
+        <v/>
+      </c>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="17">
+        <f>E36-C36+IF(G36="",F36,G36)</f>
+        <v/>
+      </c>
+      <c r="I36" s="17">
+        <f>F62*D62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="27" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B37" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C36" s="28">
-        <f>SUM('Variables_And_Log'!F10:H10)</f>
-        <v/>
-      </c>
-      <c r="D36" s="29">
-        <f>E59</f>
-        <v/>
-      </c>
-      <c r="E36" s="28">
-        <f>H35</f>
-        <v/>
-      </c>
-      <c r="F36" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D36)),MAX(0,I36-E36),0)</f>
-        <v/>
-      </c>
-      <c r="G36" s="31" t="n"/>
-      <c r="H36" s="28">
-        <f>E36-C36+IF(G36="",F36,G36)</f>
-        <v/>
-      </c>
-      <c r="I36" s="28">
-        <f>$B$2*D59</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="14" t="n">
-        <v>2033</v>
-      </c>
-      <c r="B37" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C37" s="17">
-        <f>SUM('Variables_And_Log'!I10:K10)</f>
-        <v/>
-      </c>
-      <c r="D37" s="32">
-        <f>E59</f>
-        <v/>
-      </c>
-      <c r="E37" s="17">
+      <c r="C37" s="29">
+        <f>SUM('Variables_And_Log'!F9:H9)</f>
+        <v/>
+      </c>
+      <c r="D37" s="30">
+        <f>E63</f>
+        <v/>
+      </c>
+      <c r="E37" s="29">
         <f>H36</f>
         <v/>
       </c>
-      <c r="F37" s="22">
+      <c r="F37" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D37)),MAX(0,I37-E37),0)</f>
         <v/>
       </c>
-      <c r="G37" s="18" t="n"/>
-      <c r="H37" s="17">
+      <c r="G37" s="32" t="n"/>
+      <c r="H37" s="29">
         <f>E37-C37+IF(G37="",F37,G37)</f>
         <v/>
       </c>
-      <c r="I37" s="17">
-        <f>$B$2*D59</f>
+      <c r="I37" s="29">
+        <f>F63*D63</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="14" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B38" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C38" s="17">
-        <f>SUM('Variables_And_Log'!L10:N10)</f>
-        <v/>
-      </c>
-      <c r="D38" s="32">
-        <f>E59</f>
+        <f>SUM('Variables_And_Log'!I9:K9)</f>
+        <v/>
+      </c>
+      <c r="D38" s="33">
+        <f>E63</f>
         <v/>
       </c>
       <c r="E38" s="17">
@@ -2857,25 +2746,25 @@
         <v/>
       </c>
       <c r="I38" s="17">
-        <f>$B$2*D59</f>
+        <f>F63*D63</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="14" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B39" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C39" s="17">
-        <f>SUM('Variables_And_Log'!O10:Q10)</f>
-        <v/>
-      </c>
-      <c r="D39" s="32">
-        <f>E59</f>
+        <f>SUM('Variables_And_Log'!L9:N9)</f>
+        <v/>
+      </c>
+      <c r="D39" s="33">
+        <f>E63</f>
         <v/>
       </c>
       <c r="E39" s="17">
@@ -2892,95 +2781,95 @@
         <v/>
       </c>
       <c r="I39" s="17">
-        <f>$B$2*D59</f>
+        <f>F63*D63</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="26" t="n">
-        <v>2034</v>
-      </c>
-      <c r="B40" s="27" t="inlineStr">
+      <c r="A40" s="14" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C40" s="17">
+        <f>SUM('Variables_And_Log'!O9:Q9)</f>
+        <v/>
+      </c>
+      <c r="D40" s="33">
+        <f>E63</f>
+        <v/>
+      </c>
+      <c r="E40" s="17">
+        <f>H39</f>
+        <v/>
+      </c>
+      <c r="F40" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D40)),MAX(0,I40-E40),0)</f>
+        <v/>
+      </c>
+      <c r="G40" s="18" t="n"/>
+      <c r="H40" s="17">
+        <f>E40-C40+IF(G40="",F40,G40)</f>
+        <v/>
+      </c>
+      <c r="I40" s="17">
+        <f>F63*D63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="27" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B41" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C40" s="28">
-        <f>SUM('Variables_And_Log'!F11:H11)</f>
-        <v/>
-      </c>
-      <c r="D40" s="29">
-        <f>E60</f>
-        <v/>
-      </c>
-      <c r="E40" s="28">
-        <f>H39</f>
-        <v/>
-      </c>
-      <c r="F40" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D40)),MAX(0,I40-E40),0)</f>
-        <v/>
-      </c>
-      <c r="G40" s="31" t="n"/>
-      <c r="H40" s="28">
-        <f>E40-C40+IF(G40="",F40,G40)</f>
-        <v/>
-      </c>
-      <c r="I40" s="28">
-        <f>$B$2*D60</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="14" t="n">
-        <v>2034</v>
-      </c>
-      <c r="B41" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C41" s="17">
-        <f>SUM('Variables_And_Log'!I11:K11)</f>
-        <v/>
-      </c>
-      <c r="D41" s="32">
-        <f>E60</f>
-        <v/>
-      </c>
-      <c r="E41" s="17">
+      <c r="C41" s="29">
+        <f>SUM('Variables_And_Log'!F10:H10)</f>
+        <v/>
+      </c>
+      <c r="D41" s="30">
+        <f>E64</f>
+        <v/>
+      </c>
+      <c r="E41" s="29">
         <f>H40</f>
         <v/>
       </c>
-      <c r="F41" s="22">
+      <c r="F41" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D41)),MAX(0,I41-E41),0)</f>
         <v/>
       </c>
-      <c r="G41" s="18" t="n"/>
-      <c r="H41" s="17">
+      <c r="G41" s="32" t="n"/>
+      <c r="H41" s="29">
         <f>E41-C41+IF(G41="",F41,G41)</f>
         <v/>
       </c>
-      <c r="I41" s="17">
-        <f>$B$2*D60</f>
+      <c r="I41" s="29">
+        <f>F64*D64</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="14" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B42" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C42" s="17">
-        <f>SUM('Variables_And_Log'!L11:N11)</f>
-        <v/>
-      </c>
-      <c r="D42" s="32">
-        <f>E60</f>
+        <f>SUM('Variables_And_Log'!I10:K10)</f>
+        <v/>
+      </c>
+      <c r="D42" s="33">
+        <f>E64</f>
         <v/>
       </c>
       <c r="E42" s="17">
@@ -2997,25 +2886,25 @@
         <v/>
       </c>
       <c r="I42" s="17">
-        <f>$B$2*D60</f>
+        <f>F64*D64</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="14" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B43" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C43" s="17">
-        <f>SUM('Variables_And_Log'!O11:Q11)</f>
-        <v/>
-      </c>
-      <c r="D43" s="32">
-        <f>E60</f>
+        <f>SUM('Variables_And_Log'!L10:N10)</f>
+        <v/>
+      </c>
+      <c r="D43" s="33">
+        <f>E64</f>
         <v/>
       </c>
       <c r="E43" s="17">
@@ -3032,95 +2921,95 @@
         <v/>
       </c>
       <c r="I43" s="17">
-        <f>$B$2*D60</f>
+        <f>F64*D64</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="26" t="n">
-        <v>2035</v>
-      </c>
-      <c r="B44" s="27" t="inlineStr">
+      <c r="A44" s="14" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C44" s="17">
+        <f>SUM('Variables_And_Log'!O10:Q10)</f>
+        <v/>
+      </c>
+      <c r="D44" s="33">
+        <f>E64</f>
+        <v/>
+      </c>
+      <c r="E44" s="17">
+        <f>H43</f>
+        <v/>
+      </c>
+      <c r="F44" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D44)),MAX(0,I44-E44),0)</f>
+        <v/>
+      </c>
+      <c r="G44" s="18" t="n"/>
+      <c r="H44" s="17">
+        <f>E44-C44+IF(G44="",F44,G44)</f>
+        <v/>
+      </c>
+      <c r="I44" s="17">
+        <f>F64*D64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="27" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B45" s="28" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C44" s="28">
-        <f>SUM('Variables_And_Log'!F12:H12)</f>
-        <v/>
-      </c>
-      <c r="D44" s="29">
-        <f>E61</f>
-        <v/>
-      </c>
-      <c r="E44" s="28">
-        <f>H43</f>
-        <v/>
-      </c>
-      <c r="F44" s="30">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D44)),MAX(0,I44-E44),0)</f>
-        <v/>
-      </c>
-      <c r="G44" s="31" t="n"/>
-      <c r="H44" s="28">
-        <f>E44-C44+IF(G44="",F44,G44)</f>
-        <v/>
-      </c>
-      <c r="I44" s="28">
-        <f>$B$2*D61</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="28" customHeight="1">
-      <c r="A45" s="14" t="n">
-        <v>2035</v>
-      </c>
-      <c r="B45" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C45" s="17">
-        <f>SUM('Variables_And_Log'!I12:K12)</f>
-        <v/>
-      </c>
-      <c r="D45" s="32">
-        <f>E61</f>
-        <v/>
-      </c>
-      <c r="E45" s="17">
+      <c r="C45" s="29">
+        <f>SUM('Variables_And_Log'!F11:H11)</f>
+        <v/>
+      </c>
+      <c r="D45" s="30">
+        <f>E65</f>
+        <v/>
+      </c>
+      <c r="E45" s="29">
         <f>H44</f>
         <v/>
       </c>
-      <c r="F45" s="22">
+      <c r="F45" s="31">
         <f>IF(ISNUMBER(SEARCH("GOOD",D45)),MAX(0,I45-E45),0)</f>
         <v/>
       </c>
-      <c r="G45" s="18" t="n"/>
-      <c r="H45" s="17">
+      <c r="G45" s="32" t="n"/>
+      <c r="H45" s="29">
         <f>E45-C45+IF(G45="",F45,G45)</f>
         <v/>
       </c>
-      <c r="I45" s="17">
-        <f>$B$2*D61</f>
+      <c r="I45" s="29">
+        <f>F65*D65</f>
         <v/>
       </c>
     </row>
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="14" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B46" s="20" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C46" s="17">
-        <f>SUM('Variables_And_Log'!L12:N12)</f>
-        <v/>
-      </c>
-      <c r="D46" s="32">
-        <f>E61</f>
+        <f>SUM('Variables_And_Log'!I11:K11)</f>
+        <v/>
+      </c>
+      <c r="D46" s="33">
+        <f>E65</f>
         <v/>
       </c>
       <c r="E46" s="17">
@@ -3137,25 +3026,25 @@
         <v/>
       </c>
       <c r="I46" s="17">
-        <f>$B$2*D61</f>
+        <f>F65*D65</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1">
       <c r="A47" s="14" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B47" s="20" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C47" s="17">
-        <f>SUM('Variables_And_Log'!O12:Q12)</f>
-        <v/>
-      </c>
-      <c r="D47" s="32">
-        <f>E61</f>
+        <f>SUM('Variables_And_Log'!L11:N11)</f>
+        <v/>
+      </c>
+      <c r="D47" s="33">
+        <f>E65</f>
         <v/>
       </c>
       <c r="E47" s="17">
@@ -3172,349 +3061,570 @@
         <v/>
       </c>
       <c r="I47" s="17">
-        <f>$B$2*D61</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>ANNUAL SRR HURDLE MODEL — STRATEGIC PACING CHECK (GATES THE QUARTERLY REFILL ABOVE)</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-    </row>
-    <row r="51" ht="32" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>Total Annual Hurdle Rate</t>
-        </is>
-      </c>
-      <c r="C51" s="11" t="inlineStr">
-        <is>
-          <t>Annual Outflows (W_t)</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Target Portfolio (P_track)</t>
-        </is>
-      </c>
-      <c r="E51" s="11" t="inlineStr">
-        <is>
-          <t>Performance Logic Trigger</t>
-        </is>
+        <f>F65*D65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="14" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B48" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C48" s="17">
+        <f>SUM('Variables_And_Log'!O11:Q11)</f>
+        <v/>
+      </c>
+      <c r="D48" s="33">
+        <f>E65</f>
+        <v/>
+      </c>
+      <c r="E48" s="17">
+        <f>H47</f>
+        <v/>
+      </c>
+      <c r="F48" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D48)),MAX(0,I48-E48),0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="18" t="n"/>
+      <c r="H48" s="17">
+        <f>E48-C48+IF(G48="",F48,G48)</f>
+        <v/>
+      </c>
+      <c r="I48" s="17">
+        <f>F65*D65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="27" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B49" s="28" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C49" s="29">
+        <f>SUM('Variables_And_Log'!F12:H12)</f>
+        <v/>
+      </c>
+      <c r="D49" s="30">
+        <f>E66</f>
+        <v/>
+      </c>
+      <c r="E49" s="29">
+        <f>H48</f>
+        <v/>
+      </c>
+      <c r="F49" s="31">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D49)),MAX(0,I49-E49),0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="32" t="n"/>
+      <c r="H49" s="29">
+        <f>E49-C49+IF(G49="",F49,G49)</f>
+        <v/>
+      </c>
+      <c r="I49" s="29">
+        <f>F66*D66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="14" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C50" s="17">
+        <f>SUM('Variables_And_Log'!I12:K12)</f>
+        <v/>
+      </c>
+      <c r="D50" s="33">
+        <f>E66</f>
+        <v/>
+      </c>
+      <c r="E50" s="17">
+        <f>H49</f>
+        <v/>
+      </c>
+      <c r="F50" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D50)),MAX(0,I50-E50),0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="18" t="n"/>
+      <c r="H50" s="17">
+        <f>E50-C50+IF(G50="",F50,G50)</f>
+        <v/>
+      </c>
+      <c r="I50" s="17">
+        <f>F66*D66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="14" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C51" s="17">
+        <f>SUM('Variables_And_Log'!L12:N12)</f>
+        <v/>
+      </c>
+      <c r="D51" s="33">
+        <f>E66</f>
+        <v/>
+      </c>
+      <c r="E51" s="17">
+        <f>H50</f>
+        <v/>
+      </c>
+      <c r="F51" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D51)),MAX(0,I51-E51),0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="18" t="n"/>
+      <c r="H51" s="17">
+        <f>E51-C51+IF(G51="",F51,G51)</f>
+        <v/>
+      </c>
+      <c r="I51" s="17">
+        <f>F66*D66</f>
+        <v/>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1">
       <c r="A52" s="14" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B52" s="16">
-        <f>'Variables_And_Log'!D3</f>
-        <v/>
+        <v>2035</v>
+      </c>
+      <c r="B52" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
       </c>
       <c r="C52" s="17">
-        <f>'Variables_And_Log'!E3</f>
-        <v/>
-      </c>
-      <c r="D52" s="17">
-        <f>ROUND(($B$1*B52)-C52,2)</f>
-        <v/>
-      </c>
-      <c r="E52" s="32">
-        <f>IF(B$1&gt;=D52,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="14" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B53" s="16">
-        <f>'Variables_And_Log'!D4</f>
-        <v/>
-      </c>
-      <c r="C53" s="17">
-        <f>'Variables_And_Log'!E4</f>
-        <v/>
-      </c>
-      <c r="D53" s="17">
-        <f>ROUND((D52*B53)-C53,2)</f>
-        <v/>
-      </c>
-      <c r="E53" s="32">
-        <f>IF(B$1&gt;=D53,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="14" t="n">
-        <v>2028</v>
-      </c>
-      <c r="B54" s="16">
-        <f>'Variables_And_Log'!D5</f>
-        <v/>
-      </c>
-      <c r="C54" s="17">
-        <f>'Variables_And_Log'!E5</f>
-        <v/>
-      </c>
-      <c r="D54" s="17">
-        <f>ROUND((D53*B54)-C54,2)</f>
-        <v/>
-      </c>
-      <c r="E54" s="32">
-        <f>IF(B$1&gt;=D54,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="14" t="n">
-        <v>2029</v>
-      </c>
-      <c r="B55" s="16">
-        <f>'Variables_And_Log'!D6</f>
-        <v/>
-      </c>
-      <c r="C55" s="17">
-        <f>'Variables_And_Log'!E6</f>
-        <v/>
-      </c>
-      <c r="D55" s="17">
-        <f>ROUND((D54*B55)-C55,2)</f>
-        <v/>
-      </c>
-      <c r="E55" s="32">
-        <f>IF(B$1&gt;=D55,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="14" t="n">
-        <v>2030</v>
-      </c>
-      <c r="B56" s="16">
-        <f>'Variables_And_Log'!D7</f>
-        <v/>
-      </c>
-      <c r="C56" s="17">
-        <f>'Variables_And_Log'!E7</f>
-        <v/>
-      </c>
-      <c r="D56" s="17">
-        <f>ROUND((D55*B56)-C56,2)</f>
-        <v/>
-      </c>
-      <c r="E56" s="32">
-        <f>IF(B$1&gt;=D56,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
+        <f>SUM('Variables_And_Log'!O12:Q12)</f>
+        <v/>
+      </c>
+      <c r="D52" s="33">
+        <f>E66</f>
+        <v/>
+      </c>
+      <c r="E52" s="17">
+        <f>H51</f>
+        <v/>
+      </c>
+      <c r="F52" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D52)),MAX(0,I52-E52),0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="18" t="n"/>
+      <c r="H52" s="17">
+        <f>E52-C52+IF(G52="",F52,G52)</f>
+        <v/>
+      </c>
+      <c r="I52" s="17">
+        <f>F66*D66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>ANNUAL SRR HURDLE MODEL — STRATEGIC PACING CHECK (GATES THE QUARTERLY REFILL ABOVE)</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>Total Annual Hurdle Rate</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Annual Outflows (W_t)</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Simulated Target Portfolio (P_track)</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>Performance Logic Trigger</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>Safety Anchor % (This Year)</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="14" t="n">
-        <v>2031</v>
+        <v>2026</v>
       </c>
       <c r="B57" s="16">
-        <f>'Variables_And_Log'!D8</f>
+        <f>'Variables_And_Log'!D3</f>
         <v/>
       </c>
       <c r="C57" s="17">
-        <f>'Variables_And_Log'!E8</f>
+        <f>'Variables_And_Log'!E3</f>
         <v/>
       </c>
       <c r="D57" s="17">
-        <f>ROUND((D56*B57)-C57,2)</f>
-        <v/>
-      </c>
-      <c r="E57" s="32">
+        <f>ROUND(($B$1*B57)-C57,2)</f>
+        <v/>
+      </c>
+      <c r="E57" s="33">
         <f>IF(B$1&gt;=D57,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F57" s="16">
+        <f>IF(A57-$B$2&lt;$B$4,$B$5,$B$6)</f>
         <v/>
       </c>
     </row>
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="14" t="n">
-        <v>2032</v>
+        <v>2027</v>
       </c>
       <c r="B58" s="16">
-        <f>'Variables_And_Log'!D9</f>
+        <f>'Variables_And_Log'!D4</f>
         <v/>
       </c>
       <c r="C58" s="17">
-        <f>'Variables_And_Log'!E9</f>
+        <f>'Variables_And_Log'!E4</f>
         <v/>
       </c>
       <c r="D58" s="17">
         <f>ROUND((D57*B58)-C58,2)</f>
         <v/>
       </c>
-      <c r="E58" s="32">
+      <c r="E58" s="33">
         <f>IF(B$1&gt;=D58,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F58" s="16">
+        <f>IF(A58-$B$2&lt;$B$4,$B$5,$B$6)</f>
         <v/>
       </c>
     </row>
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="14" t="n">
-        <v>2033</v>
+        <v>2028</v>
       </c>
       <c r="B59" s="16">
-        <f>'Variables_And_Log'!D10</f>
+        <f>'Variables_And_Log'!D5</f>
         <v/>
       </c>
       <c r="C59" s="17">
-        <f>'Variables_And_Log'!E10</f>
+        <f>'Variables_And_Log'!E5</f>
         <v/>
       </c>
       <c r="D59" s="17">
         <f>ROUND((D58*B59)-C59,2)</f>
         <v/>
       </c>
-      <c r="E59" s="32">
+      <c r="E59" s="33">
         <f>IF(B$1&gt;=D59,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F59" s="16">
+        <f>IF(A59-$B$2&lt;$B$4,$B$5,$B$6)</f>
         <v/>
       </c>
     </row>
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="14" t="n">
-        <v>2034</v>
+        <v>2029</v>
       </c>
       <c r="B60" s="16">
-        <f>'Variables_And_Log'!D11</f>
+        <f>'Variables_And_Log'!D6</f>
         <v/>
       </c>
       <c r="C60" s="17">
-        <f>'Variables_And_Log'!E11</f>
+        <f>'Variables_And_Log'!E6</f>
         <v/>
       </c>
       <c r="D60" s="17">
         <f>ROUND((D59*B60)-C60,2)</f>
         <v/>
       </c>
-      <c r="E60" s="32">
+      <c r="E60" s="33">
         <f>IF(B$1&gt;=D60,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F60" s="16">
+        <f>IF(A60-$B$2&lt;$B$4,$B$5,$B$6)</f>
         <v/>
       </c>
     </row>
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="14" t="n">
-        <v>2035</v>
+        <v>2030</v>
       </c>
       <c r="B61" s="16">
-        <f>'Variables_And_Log'!D12</f>
+        <f>'Variables_And_Log'!D7</f>
         <v/>
       </c>
       <c r="C61" s="17">
-        <f>'Variables_And_Log'!E12</f>
+        <f>'Variables_And_Log'!E7</f>
         <v/>
       </c>
       <c r="D61" s="17">
         <f>ROUND((D60*B61)-C61,2)</f>
         <v/>
       </c>
-      <c r="E61" s="32">
+      <c r="E61" s="33">
         <f>IF(B$1&gt;=D61,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
         <v/>
       </c>
-    </row>
-    <row r="62"/>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="F61" s="16">
+        <f>IF(A61-$B$2&lt;$B$4,$B$5,$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1">
+      <c r="A62" s="14" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B62" s="16">
+        <f>'Variables_And_Log'!D8</f>
+        <v/>
+      </c>
+      <c r="C62" s="17">
+        <f>'Variables_And_Log'!E8</f>
+        <v/>
+      </c>
+      <c r="D62" s="17">
+        <f>ROUND((D61*B62)-C62,2)</f>
+        <v/>
+      </c>
+      <c r="E62" s="33">
+        <f>IF(B$1&gt;=D62,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F62" s="16">
+        <f>IF(A62-$B$2&lt;$B$4,$B$5,$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1">
+      <c r="A63" s="14" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B63" s="16">
+        <f>'Variables_And_Log'!D9</f>
+        <v/>
+      </c>
+      <c r="C63" s="17">
+        <f>'Variables_And_Log'!E9</f>
+        <v/>
+      </c>
+      <c r="D63" s="17">
+        <f>ROUND((D62*B63)-C63,2)</f>
+        <v/>
+      </c>
+      <c r="E63" s="33">
+        <f>IF(B$1&gt;=D63,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F63" s="16">
+        <f>IF(A63-$B$2&lt;$B$4,$B$5,$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="14" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B64" s="16">
+        <f>'Variables_And_Log'!D10</f>
+        <v/>
+      </c>
+      <c r="C64" s="17">
+        <f>'Variables_And_Log'!E10</f>
+        <v/>
+      </c>
+      <c r="D64" s="17">
+        <f>ROUND((D63*B64)-C64,2)</f>
+        <v/>
+      </c>
+      <c r="E64" s="33">
+        <f>IF(B$1&gt;=D64,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F64" s="16">
+        <f>IF(A64-$B$2&lt;$B$4,$B$5,$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="28" customHeight="1">
+      <c r="A65" s="14" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B65" s="16">
+        <f>'Variables_And_Log'!D11</f>
+        <v/>
+      </c>
+      <c r="C65" s="17">
+        <f>'Variables_And_Log'!E11</f>
+        <v/>
+      </c>
+      <c r="D65" s="17">
+        <f>ROUND((D64*B65)-C65,2)</f>
+        <v/>
+      </c>
+      <c r="E65" s="33">
+        <f>IF(B$1&gt;=D65,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F65" s="16">
+        <f>IF(A65-$B$2&lt;$B$4,$B$5,$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="28" customHeight="1">
+      <c r="A66" s="14" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B66" s="16">
+        <f>'Variables_And_Log'!D12</f>
+        <v/>
+      </c>
+      <c r="C66" s="17">
+        <f>'Variables_And_Log'!E12</f>
+        <v/>
+      </c>
+      <c r="D66" s="17">
+        <f>ROUND((D65*B66)-C66,2)</f>
+        <v/>
+      </c>
+      <c r="E66" s="33">
+        <f>IF(B$1&gt;=D66,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="F66" s="16">
+        <f>IF(A66-$B$2&lt;$B$4,$B$5,$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67"/>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>EXTRA CAPACITY INDICATORS</t>
         </is>
       </c>
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="2" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="24" t="inlineStr">
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="24" t="inlineStr">
         <is>
           <t>Your Pre-Tax Rollover Conduit Capacity</t>
         </is>
       </c>
-      <c r="B64" s="17">
+      <c r="B69" s="17">
         <f>'Account_Tracker'!$C$3</f>
         <v/>
       </c>
-      <c r="C64" s="21">
-        <f>IF(B64&gt;0,"Conduit Open","Conduit Closed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65"/>
-    <row r="66">
-      <c r="A66" s="24" t="inlineStr">
+      <c r="C69" s="21">
+        <f>IF(B69&gt;0,"Conduit Open","Conduit Closed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70"/>
+    <row r="71">
+      <c r="A71" s="24" t="inlineStr">
         <is>
           <t>TSP Cash Buffer Runway (Months)</t>
         </is>
       </c>
-      <c r="B66" s="33">
+      <c r="B71" s="34">
         <f>IFERROR('Account_Tracker'!$C$2/AVERAGE('Variables_And_Log'!$F$3:$Q$3),"Log Monthly Payments to Calculate")</f>
         <v/>
       </c>
-      <c r="C66" s="21">
-        <f>IF(ISNUMBER(B66),IF(B66&gt;36,"Safe: 3+ Year Volatility Shield","Caution: Shield Shrinking"),"Awaiting Payment Data")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="19" t="inlineStr">
+      <c r="C71" s="21">
+        <f>IF(ISNUMBER(B71),IF(B71&gt;36,"Safe: 3+ Year Volatility Shield","Caution: Shield Shrinking"),"Awaiting Payment Data")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="19" t="inlineStr">
         <is>
           <t>(Runway uses the average of whichever 2026 monthly TSP payments you've logged so far.)</t>
         </is>
       </c>
-    </row>
-    <row r="68"/>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>EMERGENCY LIQUIDITY PROTOCOL — NEXT-DOLLAR PRIORITY ENGINE</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="2" t="n"/>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
-    </row>
-    <row r="70" ht="60" customHeight="1">
-      <c r="A70" s="24" t="inlineStr">
-        <is>
-          <t>Next-Dollar Liquidity Priority</t>
-        </is>
-      </c>
-      <c r="B70" s="34">
-        <f>IF('Account_Tracker'!$C$2&gt;0,"🛡️ SHIELD ACTIVE: Continue automated monthly draws directly from the TSP G Fund. Your equity engines are fully insulated from sequence-of-returns risk.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8&gt;0),"⚠️ SHIELD BROKEN: TSP G Fund is exhausted. IMMEDIATELY divert monthly checking draws to your Merrill Edge Cash Buffer. This buys next-day liquidity via Bank of America without forced retirement asset sales.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8=0,'Account_Tracker'!$C$6&gt;0),"🚨 EMERGENCY LIQUIDATION - STAGE 1: G Fund and Cash Buffers are exhausted. Turn on monthly distributions from Spouse's Current Employer 403b. Their pre-tax employer plan qualifies for the Maryland Pension Exclusion at age 65, making it more tax-efficient than touching your private traditional IRA.","💥 NUCLEAR PROTOCOL - STAGE 2: Absolute liquidity crisis. You are forced to break all shields. Begin selling shares of the 2065 Target Date Funds within your Private Traditional IRAs to fund monthly expenses. Maximize tax withholding at the time of distribution to shield your remaining capital from underpayment penalties.")))</f>
-        <v/>
-      </c>
-      <c r="C70" s="6" t="n"/>
-      <c r="D70" s="6" t="n"/>
-      <c r="E70" s="6" t="n"/>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="B71" s="6" t="n"/>
-      <c r="C71" s="6" t="n"/>
-      <c r="D71" s="6" t="n"/>
-      <c r="E71" s="6" t="n"/>
-    </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="6" t="n"/>
-      <c r="C72" s="6" t="n"/>
-      <c r="D72" s="6" t="n"/>
-      <c r="E72" s="6" t="n"/>
     </row>
     <row r="73"/>
     <row r="74">
-      <c r="A74" s="19" t="inlineStr">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>EMERGENCY LIQUIDITY PROTOCOL — NEXT-DOLLAR PRIORITY ENGINE</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n"/>
+      <c r="C74" s="2" t="n"/>
+      <c r="D74" s="2" t="n"/>
+      <c r="E74" s="2" t="n"/>
+    </row>
+    <row r="75" ht="60" customHeight="1">
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>Next-Dollar Liquidity Priority</t>
+        </is>
+      </c>
+      <c r="B75" s="35">
+        <f>IF('Account_Tracker'!$C$2&gt;0,"🛡️ SHIELD ACTIVE: Continue automated monthly draws directly from the TSP G Fund. Your equity engines are fully insulated from sequence-of-returns risk.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8&gt;0),"⚠️ SHIELD BROKEN: TSP G Fund is exhausted. IMMEDIATELY divert monthly checking draws to your Merrill Edge Cash Buffer. This buys next-day liquidity via Bank of America without forced retirement asset sales.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8=0,'Account_Tracker'!$C$6&gt;0),"🚨 EMERGENCY LIQUIDATION - STAGE 1: G Fund and Cash Buffers are exhausted. Turn on monthly distributions from Spouse's Current Employer 403b. Their pre-tax employer plan qualifies for the Maryland Pension Exclusion at age 65, making it more tax-efficient than touching your private traditional IRA.","💥 NUCLEAR PROTOCOL - STAGE 2: Absolute liquidity crisis. You are forced to break all shields. Begin selling shares of the 2065 Target Date Funds within your Private Traditional IRAs to fund monthly expenses. Maximize tax withholding at the time of distribution to shield your remaining capital from underpayment penalties.")))</f>
+        <v/>
+      </c>
+      <c r="C75" s="6" t="n"/>
+      <c r="D75" s="6" t="n"/>
+      <c r="E75" s="6" t="n"/>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="6" t="n"/>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="6" t="n"/>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="6" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="6" t="n"/>
+    </row>
+    <row r="78"/>
+    <row r="79">
+      <c r="A79" s="19" t="inlineStr">
         <is>
           <t>Legend: pale-yellow cells are yours to type into; white cells hold formulas -- please don't overwrite them.</t>
         </is>
@@ -3522,13 +3632,13 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A69:E69"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="B70:E72"/>
-    <mergeCell ref="A63:C63"/>
-    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="B75:E77"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A55:F55"/>
   </mergeCells>
-  <conditionalFormatting sqref="B70:B72">
+  <conditionalFormatting sqref="B75:B77">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>'Account_Tracker'!$C$2&gt;0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add scenario demo workbook; floor G Fund balance at zero
household_portfolio_scenario_demo.xlsx is a standalone companion sharing
the live tracker's 4-tab structure, with generic pre-filled data and a
Bear/Bull/Choppy scenario selector that simulates household wealth
forward year by year, so the Quarterly Refill Engine's GOOD/POOR trigger
visibly fires in both directions -- something the live tracker can't show
since it only ever compares a frozen snapshot. Meant to be shared with a
financial advisor and eventually posted publicly as a template.

Building it surfaced a real bug shared by both workbooks: the G Fund
"End of Quarter" balance formula had no floor, so a sustained run of POOR
years with no refill drove it deeply negative. Added a MAX(0, ...) floor
to both generators.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dyD4f3m3cXsViTiCTbG7n
</commit_message>
<xml_diff>
--- a/household_portfolio_engine.xlsx
+++ b/household_portfolio_engine.xlsx
@@ -1867,7 +1867,7 @@
       </c>
       <c r="G13" s="32" t="n"/>
       <c r="H13" s="29">
-        <f>E13-C13+IF(G13="",F13,G13)</f>
+        <f>MAX(0,E13-C13+IF(G13="",F13,G13))</f>
         <v/>
       </c>
       <c r="I13" s="29">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="G14" s="18" t="n"/>
       <c r="H14" s="17">
-        <f>E14-C14+IF(G14="",F14,G14)</f>
+        <f>MAX(0,E14-C14+IF(G14="",F14,G14))</f>
         <v/>
       </c>
       <c r="I14" s="17">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G15" s="18" t="n"/>
       <c r="H15" s="17">
-        <f>E15-C15+IF(G15="",F15,G15)</f>
+        <f>MAX(0,E15-C15+IF(G15="",F15,G15))</f>
         <v/>
       </c>
       <c r="I15" s="17">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="G16" s="18" t="n"/>
       <c r="H16" s="17">
-        <f>E16-C16+IF(G16="",F16,G16)</f>
+        <f>MAX(0,E16-C16+IF(G16="",F16,G16))</f>
         <v/>
       </c>
       <c r="I16" s="17">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G17" s="32" t="n"/>
       <c r="H17" s="29">
-        <f>E17-C17+IF(G17="",F17,G17)</f>
+        <f>MAX(0,E17-C17+IF(G17="",F17,G17))</f>
         <v/>
       </c>
       <c r="I17" s="29">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="G18" s="18" t="n"/>
       <c r="H18" s="17">
-        <f>E18-C18+IF(G18="",F18,G18)</f>
+        <f>MAX(0,E18-C18+IF(G18="",F18,G18))</f>
         <v/>
       </c>
       <c r="I18" s="17">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G19" s="18" t="n"/>
       <c r="H19" s="17">
-        <f>E19-C19+IF(G19="",F19,G19)</f>
+        <f>MAX(0,E19-C19+IF(G19="",F19,G19))</f>
         <v/>
       </c>
       <c r="I19" s="17">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="G20" s="18" t="n"/>
       <c r="H20" s="17">
-        <f>E20-C20+IF(G20="",F20,G20)</f>
+        <f>MAX(0,E20-C20+IF(G20="",F20,G20))</f>
         <v/>
       </c>
       <c r="I20" s="17">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="G21" s="32" t="n"/>
       <c r="H21" s="29">
-        <f>E21-C21+IF(G21="",F21,G21)</f>
+        <f>MAX(0,E21-C21+IF(G21="",F21,G21))</f>
         <v/>
       </c>
       <c r="I21" s="29">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="G22" s="18" t="n"/>
       <c r="H22" s="17">
-        <f>E22-C22+IF(G22="",F22,G22)</f>
+        <f>MAX(0,E22-C22+IF(G22="",F22,G22))</f>
         <v/>
       </c>
       <c r="I22" s="17">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G23" s="18" t="n"/>
       <c r="H23" s="17">
-        <f>E23-C23+IF(G23="",F23,G23)</f>
+        <f>MAX(0,E23-C23+IF(G23="",F23,G23))</f>
         <v/>
       </c>
       <c r="I23" s="17">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="G24" s="18" t="n"/>
       <c r="H24" s="17">
-        <f>E24-C24+IF(G24="",F24,G24)</f>
+        <f>MAX(0,E24-C24+IF(G24="",F24,G24))</f>
         <v/>
       </c>
       <c r="I24" s="17">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="G25" s="32" t="n"/>
       <c r="H25" s="29">
-        <f>E25-C25+IF(G25="",F25,G25)</f>
+        <f>MAX(0,E25-C25+IF(G25="",F25,G25))</f>
         <v/>
       </c>
       <c r="I25" s="29">
@@ -2322,7 +2322,7 @@
       </c>
       <c r="G26" s="18" t="n"/>
       <c r="H26" s="17">
-        <f>E26-C26+IF(G26="",F26,G26)</f>
+        <f>MAX(0,E26-C26+IF(G26="",F26,G26))</f>
         <v/>
       </c>
       <c r="I26" s="17">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="G27" s="18" t="n"/>
       <c r="H27" s="17">
-        <f>E27-C27+IF(G27="",F27,G27)</f>
+        <f>MAX(0,E27-C27+IF(G27="",F27,G27))</f>
         <v/>
       </c>
       <c r="I27" s="17">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="G28" s="18" t="n"/>
       <c r="H28" s="17">
-        <f>E28-C28+IF(G28="",F28,G28)</f>
+        <f>MAX(0,E28-C28+IF(G28="",F28,G28))</f>
         <v/>
       </c>
       <c r="I28" s="17">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G29" s="32" t="n"/>
       <c r="H29" s="29">
-        <f>E29-C29+IF(G29="",F29,G29)</f>
+        <f>MAX(0,E29-C29+IF(G29="",F29,G29))</f>
         <v/>
       </c>
       <c r="I29" s="29">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="G30" s="18" t="n"/>
       <c r="H30" s="17">
-        <f>E30-C30+IF(G30="",F30,G30)</f>
+        <f>MAX(0,E30-C30+IF(G30="",F30,G30))</f>
         <v/>
       </c>
       <c r="I30" s="17">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G31" s="18" t="n"/>
       <c r="H31" s="17">
-        <f>E31-C31+IF(G31="",F31,G31)</f>
+        <f>MAX(0,E31-C31+IF(G31="",F31,G31))</f>
         <v/>
       </c>
       <c r="I31" s="17">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="G32" s="18" t="n"/>
       <c r="H32" s="17">
-        <f>E32-C32+IF(G32="",F32,G32)</f>
+        <f>MAX(0,E32-C32+IF(G32="",F32,G32))</f>
         <v/>
       </c>
       <c r="I32" s="17">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="G33" s="32" t="n"/>
       <c r="H33" s="29">
-        <f>E33-C33+IF(G33="",F33,G33)</f>
+        <f>MAX(0,E33-C33+IF(G33="",F33,G33))</f>
         <v/>
       </c>
       <c r="I33" s="29">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="G34" s="18" t="n"/>
       <c r="H34" s="17">
-        <f>E34-C34+IF(G34="",F34,G34)</f>
+        <f>MAX(0,E34-C34+IF(G34="",F34,G34))</f>
         <v/>
       </c>
       <c r="I34" s="17">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="G35" s="18" t="n"/>
       <c r="H35" s="17">
-        <f>E35-C35+IF(G35="",F35,G35)</f>
+        <f>MAX(0,E35-C35+IF(G35="",F35,G35))</f>
         <v/>
       </c>
       <c r="I35" s="17">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="G36" s="18" t="n"/>
       <c r="H36" s="17">
-        <f>E36-C36+IF(G36="",F36,G36)</f>
+        <f>MAX(0,E36-C36+IF(G36="",F36,G36))</f>
         <v/>
       </c>
       <c r="I36" s="17">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="G37" s="32" t="n"/>
       <c r="H37" s="29">
-        <f>E37-C37+IF(G37="",F37,G37)</f>
+        <f>MAX(0,E37-C37+IF(G37="",F37,G37))</f>
         <v/>
       </c>
       <c r="I37" s="29">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="G38" s="18" t="n"/>
       <c r="H38" s="17">
-        <f>E38-C38+IF(G38="",F38,G38)</f>
+        <f>MAX(0,E38-C38+IF(G38="",F38,G38))</f>
         <v/>
       </c>
       <c r="I38" s="17">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G39" s="18" t="n"/>
       <c r="H39" s="17">
-        <f>E39-C39+IF(G39="",F39,G39)</f>
+        <f>MAX(0,E39-C39+IF(G39="",F39,G39))</f>
         <v/>
       </c>
       <c r="I39" s="17">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="G40" s="18" t="n"/>
       <c r="H40" s="17">
-        <f>E40-C40+IF(G40="",F40,G40)</f>
+        <f>MAX(0,E40-C40+IF(G40="",F40,G40))</f>
         <v/>
       </c>
       <c r="I40" s="17">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="G41" s="32" t="n"/>
       <c r="H41" s="29">
-        <f>E41-C41+IF(G41="",F41,G41)</f>
+        <f>MAX(0,E41-C41+IF(G41="",F41,G41))</f>
         <v/>
       </c>
       <c r="I41" s="29">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="G42" s="18" t="n"/>
       <c r="H42" s="17">
-        <f>E42-C42+IF(G42="",F42,G42)</f>
+        <f>MAX(0,E42-C42+IF(G42="",F42,G42))</f>
         <v/>
       </c>
       <c r="I42" s="17">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="G43" s="18" t="n"/>
       <c r="H43" s="17">
-        <f>E43-C43+IF(G43="",F43,G43)</f>
+        <f>MAX(0,E43-C43+IF(G43="",F43,G43))</f>
         <v/>
       </c>
       <c r="I43" s="17">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="G44" s="18" t="n"/>
       <c r="H44" s="17">
-        <f>E44-C44+IF(G44="",F44,G44)</f>
+        <f>MAX(0,E44-C44+IF(G44="",F44,G44))</f>
         <v/>
       </c>
       <c r="I44" s="17">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="G45" s="32" t="n"/>
       <c r="H45" s="29">
-        <f>E45-C45+IF(G45="",F45,G45)</f>
+        <f>MAX(0,E45-C45+IF(G45="",F45,G45))</f>
         <v/>
       </c>
       <c r="I45" s="29">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="G46" s="18" t="n"/>
       <c r="H46" s="17">
-        <f>E46-C46+IF(G46="",F46,G46)</f>
+        <f>MAX(0,E46-C46+IF(G46="",F46,G46))</f>
         <v/>
       </c>
       <c r="I46" s="17">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G47" s="18" t="n"/>
       <c r="H47" s="17">
-        <f>E47-C47+IF(G47="",F47,G47)</f>
+        <f>MAX(0,E47-C47+IF(G47="",F47,G47))</f>
         <v/>
       </c>
       <c r="I47" s="17">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="G48" s="18" t="n"/>
       <c r="H48" s="17">
-        <f>E48-C48+IF(G48="",F48,G48)</f>
+        <f>MAX(0,E48-C48+IF(G48="",F48,G48))</f>
         <v/>
       </c>
       <c r="I48" s="17">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="G49" s="32" t="n"/>
       <c r="H49" s="29">
-        <f>E49-C49+IF(G49="",F49,G49)</f>
+        <f>MAX(0,E49-C49+IF(G49="",F49,G49))</f>
         <v/>
       </c>
       <c r="I49" s="29">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="G50" s="18" t="n"/>
       <c r="H50" s="17">
-        <f>E50-C50+IF(G50="",F50,G50)</f>
+        <f>MAX(0,E50-C50+IF(G50="",F50,G50))</f>
         <v/>
       </c>
       <c r="I50" s="17">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="G51" s="18" t="n"/>
       <c r="H51" s="17">
-        <f>E51-C51+IF(G51="",F51,G51)</f>
+        <f>MAX(0,E51-C51+IF(G51="",F51,G51))</f>
         <v/>
       </c>
       <c r="I51" s="17">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="G52" s="18" t="n"/>
       <c r="H52" s="17">
-        <f>E52-C52+IF(G52="",F52,G52)</f>
+        <f>MAX(0,E52-C52+IF(G52="",F52,G52))</f>
         <v/>
       </c>
       <c r="I52" s="17">

</xml_diff>